<commit_message>
fix(tasmap): remove auto-close from goto input onChanged
The goto input was closing prematurely when user typed map names or coordinates. Removed the auto-close logic from onChanged callback - input now only closes on explicit submit (Enter key).
</commit_message>
<xml_diff>
--- a/assets/tasmap50k.xlsx
+++ b/assets/tasmap50k.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrian/Development/mapping/peak_bagger/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF0C8BF-BF46-CC45-999B-7E56BB63F6C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A116002-100D-B34D-92F6-34FAA08EB4F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="261">
   <si>
     <t>Series</t>
   </si>
@@ -725,9 +725,6 @@
     <t>mgrsMid</t>
   </si>
   <si>
-    <t>EN EM</t>
-  </si>
-  <si>
     <t>DN</t>
   </si>
   <si>
@@ -767,39 +764,15 @@
     <t>CN8000009999</t>
   </si>
   <si>
-    <t>CP8000019999</t>
-  </si>
-  <si>
-    <t>EP8000019999</t>
-  </si>
-  <si>
     <t>DN1999909999</t>
   </si>
   <si>
-    <t>DP1999919999</t>
-  </si>
-  <si>
-    <t>FP1999919999</t>
-  </si>
-  <si>
     <t>CM8000080000</t>
   </si>
   <si>
-    <t>CQ8000090000</t>
-  </si>
-  <si>
-    <t>EQ8000090000</t>
-  </si>
-  <si>
     <t>DM1999980000</t>
   </si>
   <si>
-    <t>DQ1999990000</t>
-  </si>
-  <si>
-    <t>FQ1999990000</t>
-  </si>
-  <si>
     <t>eastingMin</t>
   </si>
   <si>
@@ -815,7 +788,40 @@
     <t>eastingMid</t>
   </si>
   <si>
-    <t>northgMid</t>
+    <t>DM DN</t>
+  </si>
+  <si>
+    <t>DM  DN</t>
+  </si>
+  <si>
+    <t>EM EN</t>
+  </si>
+  <si>
+    <t>EQ8000019999</t>
+  </si>
+  <si>
+    <t>FQ1999919999</t>
+  </si>
+  <si>
+    <t>EP8000090000</t>
+  </si>
+  <si>
+    <t>FP1999990000</t>
+  </si>
+  <si>
+    <t>CQ8000019999</t>
+  </si>
+  <si>
+    <t>DQ1999919999</t>
+  </si>
+  <si>
+    <t>CP8000090000</t>
+  </si>
+  <si>
+    <t>DP1999990000</t>
+  </si>
+  <si>
+    <t>northingMid</t>
   </si>
 </sst>
 </file>
@@ -3419,40 +3425,40 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="F1" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="G1" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="H1" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="I1" t="s">
         <v>227</v>
       </c>
       <c r="J1" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="K1" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="L1" t="s">
+        <v>236</v>
+      </c>
+      <c r="M1" t="s">
         <v>237</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>238</v>
-      </c>
-      <c r="N1" t="s">
-        <v>239</v>
       </c>
       <c r="O1" t="s">
         <v>214</v>
       </c>
       <c r="P1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
@@ -3481,31 +3487,31 @@
         <v>214</v>
       </c>
       <c r="J2">
-        <f>MOD(E2+20000,100000)</f>
+        <f t="shared" ref="J2:J33" si="0">MOD(E2+20000,100000)</f>
         <v>40000</v>
       </c>
       <c r="K2">
-        <f>MOD(G2+15000,100000)</f>
+        <f t="shared" ref="K2:K33" si="1">MOD(G2+15000,100000)</f>
         <v>55000</v>
       </c>
       <c r="L2" t="str">
-        <f>_xlfn.CONCAT(TRIM($D2),TEXT(E2,"00000"),TEXT(H2,"00000"))</f>
+        <f t="shared" ref="L2:L47" si="2">_xlfn.CONCAT(TRIM($D2),TEXT(E2,"00000"),TEXT(H2,"00000"))</f>
         <v>BR2000069999</v>
       </c>
       <c r="M2" t="str">
-        <f>_xlfn.CONCAT(TRIM($D2),TEXT(F2,"00000"),TEXT(H2,"00000"))</f>
+        <f t="shared" ref="M2:M47" si="3">_xlfn.CONCAT(TRIM($D2),TEXT(F2,"00000"),TEXT(H2,"00000"))</f>
         <v>BR5999969999</v>
       </c>
       <c r="N2" t="str">
-        <f>_xlfn.CONCAT(TRIM($D2),TEXT(E2,"00000"),TEXT(G2,"00000"))</f>
+        <f t="shared" ref="N2:N47" si="4">_xlfn.CONCAT(TRIM($D2),TEXT(E2,"00000"),TEXT(G2,"00000"))</f>
         <v>BR2000040000</v>
       </c>
       <c r="O2" t="str">
-        <f>_xlfn.CONCAT(TRIM($D2),TEXT(F2,"00000"),TEXT(G2,"00000"))</f>
+        <f t="shared" ref="O2:O47" si="5">_xlfn.CONCAT(TRIM($D2),TEXT(F2,"00000"),TEXT(G2,"00000"))</f>
         <v>BR5999940000</v>
       </c>
       <c r="P2">
-        <f>LEN(TRIM(D2))</f>
+        <f t="shared" ref="P2:P33" si="6">LEN(TRIM(D2))</f>
         <v>2</v>
       </c>
     </row>
@@ -3535,31 +3541,31 @@
         <v>213</v>
       </c>
       <c r="J3">
-        <f>MOD(E3+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>40000</v>
       </c>
       <c r="K3">
-        <f>MOD(G3+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>15000</v>
       </c>
       <c r="L3" t="str">
-        <f>_xlfn.CONCAT(TRIM($D3),TEXT(E3,"00000"),TEXT(H3,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>BS2000029999</v>
       </c>
       <c r="M3" t="str">
-        <f>_xlfn.CONCAT(TRIM($D3),TEXT(F3,"00000"),TEXT(H3,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>BS5999929999</v>
       </c>
       <c r="N3" t="str">
-        <f>_xlfn.CONCAT(TRIM($D3),TEXT(E3,"00000"),TEXT(G3,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>BS2000000000</v>
       </c>
       <c r="O3" t="str">
-        <f>_xlfn.CONCAT(TRIM($D3),TEXT(F3,"00000"),TEXT(G3,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>BS5999900000</v>
       </c>
       <c r="P3">
-        <f>LEN(TRIM(D3))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -3589,31 +3595,31 @@
         <v>219</v>
       </c>
       <c r="J4">
-        <f>MOD(E4+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="K4">
-        <f>MOD(G4+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>85000</v>
       </c>
       <c r="L4" t="str">
-        <f>_xlfn.CONCAT(TRIM($D4),TEXT(E4,"00000"),TEXT(H4,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>CN4000099999</v>
       </c>
       <c r="M4" t="str">
-        <f>_xlfn.CONCAT(TRIM($D4),TEXT(F4,"00000"),TEXT(H4,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>CN7999999999</v>
       </c>
       <c r="N4" t="str">
-        <f>_xlfn.CONCAT(TRIM($D4),TEXT(E4,"00000"),TEXT(G4,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>CN4000070000</v>
       </c>
       <c r="O4" t="str">
-        <f>_xlfn.CONCAT(TRIM($D4),TEXT(F4,"00000"),TEXT(G4,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>CN7999970000</v>
       </c>
       <c r="P4">
-        <f>LEN(TRIM(D4))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -3646,31 +3652,31 @@
         <v>224</v>
       </c>
       <c r="J5">
-        <f>MOD(E5+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="K5">
-        <f>MOD(G5+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>75000</v>
       </c>
       <c r="L5" t="str">
-        <f>_xlfn.CONCAT(TRIM($D5),TEXT(E5,"00000"),TEXT(H5,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>CP4000089999</v>
       </c>
       <c r="M5" t="str">
-        <f>_xlfn.CONCAT(TRIM($D5),TEXT(F5,"00000"),TEXT(H5,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>CP7999989999</v>
       </c>
       <c r="N5" t="str">
-        <f>_xlfn.CONCAT(TRIM($D5),TEXT(E5,"00000"),TEXT(G5,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>CP4000060000</v>
       </c>
       <c r="O5" t="str">
-        <f>_xlfn.CONCAT(TRIM($D5),TEXT(F5,"00000"),TEXT(G5,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>CP7999960000</v>
       </c>
       <c r="P5">
-        <f>LEN(TRIM(D5))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -3703,31 +3709,31 @@
         <v>224</v>
       </c>
       <c r="J6">
-        <f>MOD(E6+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="K6">
-        <f>MOD(G6+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>45000</v>
       </c>
       <c r="L6" t="str">
-        <f>_xlfn.CONCAT(TRIM($D6),TEXT(E6,"00000"),TEXT(H6,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>CP4000059999</v>
       </c>
       <c r="M6" t="str">
-        <f>_xlfn.CONCAT(TRIM($D6),TEXT(F6,"00000"),TEXT(H6,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>CP7999959999</v>
       </c>
       <c r="N6" t="str">
-        <f>_xlfn.CONCAT(TRIM($D6),TEXT(E6,"00000"),TEXT(G6,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>CP4000030000</v>
       </c>
       <c r="O6" t="str">
-        <f>_xlfn.CONCAT(TRIM($D6),TEXT(F6,"00000"),TEXT(G6,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>CP7999930000</v>
       </c>
       <c r="P6">
-        <f>LEN(TRIM(D6))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -3760,31 +3766,31 @@
         <v>224</v>
       </c>
       <c r="J7">
-        <f>MOD(E7+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="K7">
-        <f>MOD(G7+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>15000</v>
       </c>
       <c r="L7" t="str">
-        <f>_xlfn.CONCAT(TRIM($D7),TEXT(E7,"00000"),TEXT(H7,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>CP4000029999</v>
       </c>
       <c r="M7" t="str">
-        <f>_xlfn.CONCAT(TRIM($D7),TEXT(F7,"00000"),TEXT(H7,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>CP7999929999</v>
       </c>
       <c r="N7" t="str">
-        <f>_xlfn.CONCAT(TRIM($D7),TEXT(E7,"00000"),TEXT(G7,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>CP4000000000</v>
       </c>
       <c r="O7" t="str">
-        <f>_xlfn.CONCAT(TRIM($D7),TEXT(F7,"00000"),TEXT(G7,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>CP7999900000</v>
       </c>
       <c r="P7">
-        <f>LEN(TRIM(D7))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -3817,31 +3823,31 @@
         <v>218</v>
       </c>
       <c r="J8">
-        <f>MOD(E8+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>20000</v>
       </c>
       <c r="K8">
-        <f>MOD(G8+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>65000</v>
       </c>
       <c r="L8" t="str">
-        <f>_xlfn.CONCAT(TRIM($D8),TEXT(E8,"00000"),TEXT(H8,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>CQ0000079999</v>
       </c>
       <c r="M8" t="str">
-        <f>_xlfn.CONCAT(TRIM($D8),TEXT(F8,"00000"),TEXT(H8,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>CQ3999979999</v>
       </c>
       <c r="N8" t="str">
-        <f>_xlfn.CONCAT(TRIM($D8),TEXT(E8,"00000"),TEXT(G8,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>CQ0000050000</v>
       </c>
       <c r="O8" t="str">
-        <f>_xlfn.CONCAT(TRIM($D8),TEXT(F8,"00000"),TEXT(G8,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>CQ3999950000</v>
       </c>
       <c r="P8">
-        <f>LEN(TRIM(D8))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -3874,31 +3880,31 @@
         <v>218</v>
       </c>
       <c r="J9">
-        <f>MOD(E9+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>20000</v>
       </c>
       <c r="K9">
-        <f>MOD(G9+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>35000</v>
       </c>
       <c r="L9" t="str">
-        <f>_xlfn.CONCAT(TRIM($D9),TEXT(E9,"00000"),TEXT(H9,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>CQ0000049999</v>
       </c>
       <c r="M9" t="str">
-        <f>_xlfn.CONCAT(TRIM($D9),TEXT(F9,"00000"),TEXT(H9,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>CQ3999949999</v>
       </c>
       <c r="N9" t="str">
-        <f>_xlfn.CONCAT(TRIM($D9),TEXT(E9,"00000"),TEXT(G9,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>CQ0000020000</v>
       </c>
       <c r="O9" t="str">
-        <f>_xlfn.CONCAT(TRIM($D9),TEXT(F9,"00000"),TEXT(G9,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>CQ3999920000</v>
       </c>
       <c r="P9">
-        <f>LEN(TRIM(D9))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -3928,31 +3934,31 @@
         <v>218</v>
       </c>
       <c r="J10">
-        <f>MOD(E10+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="K10">
-        <f>MOD(G10+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>65000</v>
       </c>
       <c r="L10" t="str">
-        <f>_xlfn.CONCAT(TRIM($D10),TEXT(E10,"00000"),TEXT(H10,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>CQ4000079999</v>
       </c>
       <c r="M10" t="str">
-        <f>_xlfn.CONCAT(TRIM($D10),TEXT(F10,"00000"),TEXT(H10,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>CQ7999979999</v>
       </c>
       <c r="N10" t="str">
-        <f>_xlfn.CONCAT(TRIM($D10),TEXT(E10,"00000"),TEXT(G10,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>CQ4000050000</v>
       </c>
       <c r="O10" t="str">
-        <f>_xlfn.CONCAT(TRIM($D10),TEXT(F10,"00000"),TEXT(G10,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>CQ7999950000</v>
       </c>
       <c r="P10">
-        <f>LEN(TRIM(D10))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -3985,31 +3991,31 @@
         <v>218</v>
       </c>
       <c r="J11">
-        <f>MOD(E11+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="K11">
-        <f>MOD(G11+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>35000</v>
       </c>
       <c r="L11" t="str">
-        <f>_xlfn.CONCAT(TRIM($D11),TEXT(E11,"00000"),TEXT(H11,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>CQ4000049999</v>
       </c>
       <c r="M11" t="str">
-        <f>_xlfn.CONCAT(TRIM($D11),TEXT(F11,"00000"),TEXT(H11,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>CQ7999949999</v>
       </c>
       <c r="N11" t="str">
-        <f>_xlfn.CONCAT(TRIM($D11),TEXT(E11,"00000"),TEXT(G11,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>CQ4000020000</v>
       </c>
       <c r="O11" t="str">
-        <f>_xlfn.CONCAT(TRIM($D11),TEXT(F11,"00000"),TEXT(G11,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>CQ7999920000</v>
       </c>
       <c r="P11">
-        <f>LEN(TRIM(D11))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4039,31 +4045,31 @@
         <v>215</v>
       </c>
       <c r="J12">
-        <f>MOD(E12+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>20000</v>
       </c>
       <c r="K12">
-        <f>MOD(G12+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>25000</v>
       </c>
       <c r="L12" t="str">
-        <f>_xlfn.CONCAT(TRIM($D12),TEXT(E12,"00000"),TEXT(H12,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>CR0000039999</v>
       </c>
       <c r="M12" t="str">
-        <f>_xlfn.CONCAT(TRIM($D12),TEXT(F12,"00000"),TEXT(H12,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>CR3999939999</v>
       </c>
       <c r="N12" t="str">
-        <f>_xlfn.CONCAT(TRIM($D12),TEXT(E12,"00000"),TEXT(G12,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>CR0000010000</v>
       </c>
       <c r="O12" t="str">
-        <f>_xlfn.CONCAT(TRIM($D12),TEXT(F12,"00000"),TEXT(G12,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>CR3999910000</v>
       </c>
       <c r="P12">
-        <f>LEN(TRIM(D12))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4096,31 +4102,31 @@
         <v>221</v>
       </c>
       <c r="J13">
-        <f>MOD(E13+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>40000</v>
       </c>
       <c r="K13">
-        <f>MOD(G13+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>65000</v>
       </c>
       <c r="L13" t="str">
-        <f>_xlfn.CONCAT(TRIM($D13),TEXT(E13,"00000"),TEXT(H13,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DM2000079999</v>
       </c>
       <c r="M13" t="str">
-        <f>_xlfn.CONCAT(TRIM($D13),TEXT(F13,"00000"),TEXT(H13,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DM5999979999</v>
       </c>
       <c r="N13" t="str">
-        <f>_xlfn.CONCAT(TRIM($D13),TEXT(E13,"00000"),TEXT(G13,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DM2000050000</v>
       </c>
       <c r="O13" t="str">
-        <f>_xlfn.CONCAT(TRIM($D13),TEXT(F13,"00000"),TEXT(G13,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DM5999950000</v>
       </c>
       <c r="P13">
-        <f>LEN(TRIM(D13))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4150,34 +4156,34 @@
         <v>99999</v>
       </c>
       <c r="I14" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J14">
-        <f>MOD(E14+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>40000</v>
       </c>
       <c r="K14">
-        <f>MOD(G14+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>85000</v>
       </c>
       <c r="L14" t="str">
-        <f>_xlfn.CONCAT(TRIM($D14),TEXT(E14,"00000"),TEXT(H14,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DN2000099999</v>
       </c>
       <c r="M14" t="str">
-        <f>_xlfn.CONCAT(TRIM($D14),TEXT(F14,"00000"),TEXT(H14,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DN5999999999</v>
       </c>
       <c r="N14" t="str">
-        <f>_xlfn.CONCAT(TRIM($D14),TEXT(E14,"00000"),TEXT(G14,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DN2000070000</v>
       </c>
       <c r="O14" t="str">
-        <f>_xlfn.CONCAT(TRIM($D14),TEXT(F14,"00000"),TEXT(G14,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DN5999970000</v>
       </c>
       <c r="P14">
-        <f>LEN(TRIM(D14))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4207,34 +4213,34 @@
         <v>69999</v>
       </c>
       <c r="I15" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J15">
-        <f>MOD(E15+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>40000</v>
       </c>
       <c r="K15">
-        <f>MOD(G15+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>55000</v>
       </c>
       <c r="L15" t="str">
-        <f>_xlfn.CONCAT(TRIM($D15),TEXT(E15,"00000"),TEXT(H15,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DN2000069999</v>
       </c>
       <c r="M15" t="str">
-        <f>_xlfn.CONCAT(TRIM($D15),TEXT(F15,"00000"),TEXT(H15,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DN5999969999</v>
       </c>
       <c r="N15" t="str">
-        <f>_xlfn.CONCAT(TRIM($D15),TEXT(E15,"00000"),TEXT(G15,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DN2000040000</v>
       </c>
       <c r="O15" t="str">
-        <f>_xlfn.CONCAT(TRIM($D15),TEXT(F15,"00000"),TEXT(G15,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DN5999940000</v>
       </c>
       <c r="P15">
-        <f>LEN(TRIM(D15))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4264,34 +4270,34 @@
         <v>39999</v>
       </c>
       <c r="I16" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J16">
-        <f>MOD(E16+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>40000</v>
       </c>
       <c r="K16">
-        <f>MOD(G16+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>25000</v>
       </c>
       <c r="L16" t="str">
-        <f>_xlfn.CONCAT(TRIM($D16),TEXT(E16,"00000"),TEXT(H16,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DN2000039999</v>
       </c>
       <c r="M16" t="str">
-        <f>_xlfn.CONCAT(TRIM($D16),TEXT(F16,"00000"),TEXT(H16,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DN5999939999</v>
       </c>
       <c r="N16" t="str">
-        <f>_xlfn.CONCAT(TRIM($D16),TEXT(E16,"00000"),TEXT(G16,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DN2000010000</v>
       </c>
       <c r="O16" t="str">
-        <f>_xlfn.CONCAT(TRIM($D16),TEXT(F16,"00000"),TEXT(G16,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DN5999910000</v>
       </c>
       <c r="P16">
-        <f>LEN(TRIM(D16))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4321,34 +4327,34 @@
         <v>99999</v>
       </c>
       <c r="I17" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J17">
-        <f>MOD(E17+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>80000</v>
       </c>
       <c r="K17">
-        <f>MOD(G17+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>85000</v>
       </c>
       <c r="L17" t="str">
-        <f>_xlfn.CONCAT(TRIM($D17),TEXT(E17,"00000"),TEXT(H17,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DN6000099999</v>
       </c>
       <c r="M17" t="str">
-        <f>_xlfn.CONCAT(TRIM($D17),TEXT(F17,"00000"),TEXT(H17,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DN9999999999</v>
       </c>
       <c r="N17" t="str">
-        <f>_xlfn.CONCAT(TRIM($D17),TEXT(E17,"00000"),TEXT(G17,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DN6000070000</v>
       </c>
       <c r="O17" t="str">
-        <f>_xlfn.CONCAT(TRIM($D17),TEXT(F17,"00000"),TEXT(G17,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DN9999970000</v>
       </c>
       <c r="P17">
-        <f>LEN(TRIM(D17))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4378,34 +4384,34 @@
         <v>69999</v>
       </c>
       <c r="I18" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J18">
-        <f>MOD(E18+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>80000</v>
       </c>
       <c r="K18">
-        <f>MOD(G18+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>55000</v>
       </c>
       <c r="L18" t="str">
-        <f>_xlfn.CONCAT(TRIM($D18),TEXT(E18,"00000"),TEXT(H18,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DN6000069999</v>
       </c>
       <c r="M18" t="str">
-        <f>_xlfn.CONCAT(TRIM($D18),TEXT(F18,"00000"),TEXT(H18,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DN9999969999</v>
       </c>
       <c r="N18" t="str">
-        <f>_xlfn.CONCAT(TRIM($D18),TEXT(E18,"00000"),TEXT(G18,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DN6000040000</v>
       </c>
       <c r="O18" t="str">
-        <f>_xlfn.CONCAT(TRIM($D18),TEXT(F18,"00000"),TEXT(G18,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DN9999940000</v>
       </c>
       <c r="P18">
-        <f>LEN(TRIM(D18))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4435,34 +4441,34 @@
         <v>39999</v>
       </c>
       <c r="I19" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J19">
-        <f>MOD(E19+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>80000</v>
       </c>
       <c r="K19">
-        <f>MOD(G19+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>25000</v>
       </c>
       <c r="L19" t="str">
-        <f>_xlfn.CONCAT(TRIM($D19),TEXT(E19,"00000"),TEXT(H19,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DN6000039999</v>
       </c>
       <c r="M19" t="str">
-        <f>_xlfn.CONCAT(TRIM($D19),TEXT(F19,"00000"),TEXT(H19,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DN9999939999</v>
       </c>
       <c r="N19" t="str">
-        <f>_xlfn.CONCAT(TRIM($D19),TEXT(E19,"00000"),TEXT(G19,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DN6000010000</v>
       </c>
       <c r="O19" t="str">
-        <f>_xlfn.CONCAT(TRIM($D19),TEXT(F19,"00000"),TEXT(G19,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DN9999910000</v>
       </c>
       <c r="P19">
-        <f>LEN(TRIM(D19))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4495,31 +4501,31 @@
         <v>222</v>
       </c>
       <c r="J20">
-        <f>MOD(E20+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>40000</v>
       </c>
       <c r="K20">
-        <f>MOD(G20+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>75000</v>
       </c>
       <c r="L20" t="str">
-        <f>_xlfn.CONCAT(TRIM($D20),TEXT(E20,"00000"),TEXT(H20,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DP2000089999</v>
       </c>
       <c r="M20" t="str">
-        <f>_xlfn.CONCAT(TRIM($D20),TEXT(F20,"00000"),TEXT(H20,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DP5999989999</v>
       </c>
       <c r="N20" t="str">
-        <f>_xlfn.CONCAT(TRIM($D20),TEXT(E20,"00000"),TEXT(G20,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DP2000060000</v>
       </c>
       <c r="O20" t="str">
-        <f>_xlfn.CONCAT(TRIM($D20),TEXT(F20,"00000"),TEXT(G20,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DP5999960000</v>
       </c>
       <c r="P20">
-        <f>LEN(TRIM(D20))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4552,31 +4558,31 @@
         <v>222</v>
       </c>
       <c r="J21">
-        <f>MOD(E21+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>40000</v>
       </c>
       <c r="K21">
-        <f>MOD(G21+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>45000</v>
       </c>
       <c r="L21" t="str">
-        <f>_xlfn.CONCAT(TRIM($D21),TEXT(E21,"00000"),TEXT(H21,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DP2000059999</v>
       </c>
       <c r="M21" t="str">
-        <f>_xlfn.CONCAT(TRIM($D21),TEXT(F21,"00000"),TEXT(H21,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DP5999959999</v>
       </c>
       <c r="N21" t="str">
-        <f>_xlfn.CONCAT(TRIM($D21),TEXT(E21,"00000"),TEXT(G21,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DP2000030000</v>
       </c>
       <c r="O21" t="str">
-        <f>_xlfn.CONCAT(TRIM($D21),TEXT(F21,"00000"),TEXT(G21,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DP5999930000</v>
       </c>
       <c r="P21">
-        <f>LEN(TRIM(D21))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4609,31 +4615,31 @@
         <v>222</v>
       </c>
       <c r="J22">
-        <f>MOD(E22+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>40000</v>
       </c>
       <c r="K22">
-        <f>MOD(G22+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>15000</v>
       </c>
       <c r="L22" t="str">
-        <f>_xlfn.CONCAT(TRIM($D22),TEXT(E22,"00000"),TEXT(H22,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DP2000029999</v>
       </c>
       <c r="M22" t="str">
-        <f>_xlfn.CONCAT(TRIM($D22),TEXT(F22,"00000"),TEXT(H22,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DP5999929999</v>
       </c>
       <c r="N22" t="str">
-        <f>_xlfn.CONCAT(TRIM($D22),TEXT(E22,"00000"),TEXT(G22,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DP2000000000</v>
       </c>
       <c r="O22" t="str">
-        <f>_xlfn.CONCAT(TRIM($D22),TEXT(F22,"00000"),TEXT(G22,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DP5999900000</v>
       </c>
       <c r="P22">
-        <f>LEN(TRIM(D22))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4666,31 +4672,31 @@
         <v>222</v>
       </c>
       <c r="J23">
-        <f>MOD(E23+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>80000</v>
       </c>
       <c r="K23">
-        <f>MOD(G23+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>75000</v>
       </c>
       <c r="L23" t="str">
-        <f>_xlfn.CONCAT(TRIM($D23),TEXT(E23,"00000"),TEXT(H23,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DP6000089999</v>
       </c>
       <c r="M23" t="str">
-        <f>_xlfn.CONCAT(TRIM($D23),TEXT(F23,"00000"),TEXT(H23,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DP9999989999</v>
       </c>
       <c r="N23" t="str">
-        <f>_xlfn.CONCAT(TRIM($D23),TEXT(E23,"00000"),TEXT(G23,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DP6000060000</v>
       </c>
       <c r="O23" t="str">
-        <f>_xlfn.CONCAT(TRIM($D23),TEXT(F23,"00000"),TEXT(G23,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DP9999960000</v>
       </c>
       <c r="P23">
-        <f>LEN(TRIM(D23))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4723,31 +4729,31 @@
         <v>222</v>
       </c>
       <c r="J24">
-        <f>MOD(E24+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>80000</v>
       </c>
       <c r="K24">
-        <f>MOD(G24+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>45000</v>
       </c>
       <c r="L24" t="str">
-        <f>_xlfn.CONCAT(TRIM($D24),TEXT(E24,"00000"),TEXT(H24,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DP6000059999</v>
       </c>
       <c r="M24" t="str">
-        <f>_xlfn.CONCAT(TRIM($D24),TEXT(F24,"00000"),TEXT(H24,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DP9999959999</v>
       </c>
       <c r="N24" t="str">
-        <f>_xlfn.CONCAT(TRIM($D24),TEXT(E24,"00000"),TEXT(G24,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DP6000030000</v>
       </c>
       <c r="O24" t="str">
-        <f>_xlfn.CONCAT(TRIM($D24),TEXT(F24,"00000"),TEXT(G24,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DP9999930000</v>
       </c>
       <c r="P24">
-        <f>LEN(TRIM(D24))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4780,31 +4786,31 @@
         <v>222</v>
       </c>
       <c r="J25">
-        <f>MOD(E25+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>80000</v>
       </c>
       <c r="K25">
-        <f>MOD(G25+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>15000</v>
       </c>
       <c r="L25" t="str">
-        <f>_xlfn.CONCAT(TRIM($D25),TEXT(E25,"00000"),TEXT(H25,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DP6000029999</v>
       </c>
       <c r="M25" t="str">
-        <f>_xlfn.CONCAT(TRIM($D25),TEXT(F25,"00000"),TEXT(H25,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DP9999929999</v>
       </c>
       <c r="N25" t="str">
-        <f>_xlfn.CONCAT(TRIM($D25),TEXT(E25,"00000"),TEXT(G25,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DP6000000000</v>
       </c>
       <c r="O25" t="str">
-        <f>_xlfn.CONCAT(TRIM($D25),TEXT(F25,"00000"),TEXT(G25,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DP9999900000</v>
       </c>
       <c r="P25">
-        <f>LEN(TRIM(D25))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4837,31 +4843,31 @@
         <v>226</v>
       </c>
       <c r="J26">
-        <f>MOD(E26+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>40000</v>
       </c>
       <c r="K26">
-        <f>MOD(G26+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>35000</v>
       </c>
       <c r="L26" t="str">
-        <f>_xlfn.CONCAT(TRIM($D26),TEXT(E26,"00000"),TEXT(H26,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DQ2000049999</v>
       </c>
       <c r="M26" t="str">
-        <f>_xlfn.CONCAT(TRIM($D26),TEXT(F26,"00000"),TEXT(H26,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DQ5999949999</v>
       </c>
       <c r="N26" t="str">
-        <f>_xlfn.CONCAT(TRIM($D26),TEXT(E26,"00000"),TEXT(G26,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DQ2000020000</v>
       </c>
       <c r="O26" t="str">
-        <f>_xlfn.CONCAT(TRIM($D26),TEXT(F26,"00000"),TEXT(G26,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DQ5999920000</v>
       </c>
       <c r="P26">
-        <f>LEN(TRIM(D26))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4891,31 +4897,31 @@
         <v>226</v>
       </c>
       <c r="J27">
-        <f>MOD(E27+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>80000</v>
       </c>
       <c r="K27">
-        <f>MOD(G27+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>65000</v>
       </c>
       <c r="L27" t="str">
-        <f>_xlfn.CONCAT(TRIM($D27),TEXT(E27,"00000"),TEXT(H27,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DQ6000079999</v>
       </c>
       <c r="M27" t="str">
-        <f>_xlfn.CONCAT(TRIM($D27),TEXT(F27,"00000"),TEXT(H27,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DQ9999979999</v>
       </c>
       <c r="N27" t="str">
-        <f>_xlfn.CONCAT(TRIM($D27),TEXT(E27,"00000"),TEXT(G27,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DQ6000050000</v>
       </c>
       <c r="O27" t="str">
-        <f>_xlfn.CONCAT(TRIM($D27),TEXT(F27,"00000"),TEXT(G27,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DQ9999950000</v>
       </c>
       <c r="P27">
-        <f>LEN(TRIM(D27))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -4948,31 +4954,31 @@
         <v>226</v>
       </c>
       <c r="J28">
-        <f>MOD(E28+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>80000</v>
       </c>
       <c r="K28">
-        <f>MOD(G28+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>35000</v>
       </c>
       <c r="L28" t="str">
-        <f>_xlfn.CONCAT(TRIM($D28),TEXT(E28,"00000"),TEXT(H28,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>DQ6000049999</v>
       </c>
       <c r="M28" t="str">
-        <f>_xlfn.CONCAT(TRIM($D28),TEXT(F28,"00000"),TEXT(H28,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>DQ9999949999</v>
       </c>
       <c r="N28" t="str">
-        <f>_xlfn.CONCAT(TRIM($D28),TEXT(E28,"00000"),TEXT(G28,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>DQ6000020000</v>
       </c>
       <c r="O28" t="str">
-        <f>_xlfn.CONCAT(TRIM($D28),TEXT(F28,"00000"),TEXT(G28,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>DQ9999920000</v>
       </c>
       <c r="P28">
-        <f>LEN(TRIM(D28))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -5002,34 +5008,34 @@
         <v>99999</v>
       </c>
       <c r="I29" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J29">
-        <f>MOD(E29+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>20000</v>
       </c>
       <c r="K29">
-        <f>MOD(G29+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>85000</v>
       </c>
       <c r="L29" t="str">
-        <f>_xlfn.CONCAT(TRIM($D29),TEXT(E29,"00000"),TEXT(H29,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EN0000099999</v>
       </c>
       <c r="M29" t="str">
-        <f>_xlfn.CONCAT(TRIM($D29),TEXT(F29,"00000"),TEXT(H29,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EN3999999999</v>
       </c>
       <c r="N29" t="str">
-        <f>_xlfn.CONCAT(TRIM($D29),TEXT(E29,"00000"),TEXT(G29,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EN0000070000</v>
       </c>
       <c r="O29" t="str">
-        <f>_xlfn.CONCAT(TRIM($D29),TEXT(F29,"00000"),TEXT(G29,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EN3999970000</v>
       </c>
       <c r="P29">
-        <f>LEN(TRIM(D29))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -5059,34 +5065,34 @@
         <v>69999</v>
       </c>
       <c r="I30" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J30">
-        <f>MOD(E30+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>20000</v>
       </c>
       <c r="K30">
-        <f>MOD(G30+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>55000</v>
       </c>
       <c r="L30" t="str">
-        <f>_xlfn.CONCAT(TRIM($D30),TEXT(E30,"00000"),TEXT(H30,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EN0000069999</v>
       </c>
       <c r="M30" t="str">
-        <f>_xlfn.CONCAT(TRIM($D30),TEXT(F30,"00000"),TEXT(H30,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EN3999969999</v>
       </c>
       <c r="N30" t="str">
-        <f>_xlfn.CONCAT(TRIM($D30),TEXT(E30,"00000"),TEXT(G30,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EN0000040000</v>
       </c>
       <c r="O30" t="str">
-        <f>_xlfn.CONCAT(TRIM($D30),TEXT(F30,"00000"),TEXT(G30,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EN3999940000</v>
       </c>
       <c r="P30">
-        <f>LEN(TRIM(D30))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -5116,34 +5122,34 @@
         <v>39999</v>
       </c>
       <c r="I31" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J31">
-        <f>MOD(E31+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>20000</v>
       </c>
       <c r="K31">
-        <f>MOD(G31+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>25000</v>
       </c>
       <c r="L31" t="str">
-        <f>_xlfn.CONCAT(TRIM($D31),TEXT(E31,"00000"),TEXT(H31,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EN0000039999</v>
       </c>
       <c r="M31" t="str">
-        <f>_xlfn.CONCAT(TRIM($D31),TEXT(F31,"00000"),TEXT(H31,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EN3999939999</v>
       </c>
       <c r="N31" t="str">
-        <f>_xlfn.CONCAT(TRIM($D31),TEXT(E31,"00000"),TEXT(G31,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EN0000010000</v>
       </c>
       <c r="O31" t="str">
-        <f>_xlfn.CONCAT(TRIM($D31),TEXT(F31,"00000"),TEXT(G31,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EN3999910000</v>
       </c>
       <c r="P31">
-        <f>LEN(TRIM(D31))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -5173,34 +5179,34 @@
         <v>99999</v>
       </c>
       <c r="I32" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J32">
-        <f>MOD(E32+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="K32">
-        <f>MOD(G32+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>85000</v>
       </c>
       <c r="L32" t="str">
-        <f>_xlfn.CONCAT(TRIM($D32),TEXT(E32,"00000"),TEXT(H32,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EN4000099999</v>
       </c>
       <c r="M32" t="str">
-        <f>_xlfn.CONCAT(TRIM($D32),TEXT(F32,"00000"),TEXT(H32,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EN7999999999</v>
       </c>
       <c r="N32" t="str">
-        <f>_xlfn.CONCAT(TRIM($D32),TEXT(E32,"00000"),TEXT(G32,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EN4000070000</v>
       </c>
       <c r="O32" t="str">
-        <f>_xlfn.CONCAT(TRIM($D32),TEXT(F32,"00000"),TEXT(G32,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EN7999970000</v>
       </c>
       <c r="P32">
-        <f>LEN(TRIM(D32))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -5230,34 +5236,34 @@
         <v>69999</v>
       </c>
       <c r="I33" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J33">
-        <f>MOD(E33+20000,100000)</f>
+        <f t="shared" si="0"/>
         <v>60000</v>
       </c>
       <c r="K33">
-        <f>MOD(G33+15000,100000)</f>
+        <f t="shared" si="1"/>
         <v>55000</v>
       </c>
       <c r="L33" t="str">
-        <f>_xlfn.CONCAT(TRIM($D33),TEXT(E33,"00000"),TEXT(H33,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EN4000069999</v>
       </c>
       <c r="M33" t="str">
-        <f>_xlfn.CONCAT(TRIM($D33),TEXT(F33,"00000"),TEXT(H33,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EN7999969999</v>
       </c>
       <c r="N33" t="str">
-        <f>_xlfn.CONCAT(TRIM($D33),TEXT(E33,"00000"),TEXT(G33,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EN4000040000</v>
       </c>
       <c r="O33" t="str">
-        <f>_xlfn.CONCAT(TRIM($D33),TEXT(F33,"00000"),TEXT(G33,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EN7999940000</v>
       </c>
       <c r="P33">
-        <f>LEN(TRIM(D33))</f>
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
     </row>
@@ -5287,34 +5293,34 @@
         <v>39999</v>
       </c>
       <c r="I34" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="J34">
-        <f>MOD(E34+20000,100000)</f>
+        <f t="shared" ref="J34:J65" si="7">MOD(E34+20000,100000)</f>
         <v>60000</v>
       </c>
       <c r="K34">
-        <f>MOD(G34+15000,100000)</f>
+        <f t="shared" ref="K34:K65" si="8">MOD(G34+15000,100000)</f>
         <v>25000</v>
       </c>
       <c r="L34" t="str">
-        <f>_xlfn.CONCAT(TRIM($D34),TEXT(E34,"00000"),TEXT(H34,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EN4000039999</v>
       </c>
       <c r="M34" t="str">
-        <f>_xlfn.CONCAT(TRIM($D34),TEXT(F34,"00000"),TEXT(H34,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EN7999939999</v>
       </c>
       <c r="N34" t="str">
-        <f>_xlfn.CONCAT(TRIM($D34),TEXT(E34,"00000"),TEXT(G34,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EN4000010000</v>
       </c>
       <c r="O34" t="str">
-        <f>_xlfn.CONCAT(TRIM($D34),TEXT(F34,"00000"),TEXT(G34,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EN7999910000</v>
       </c>
       <c r="P34">
-        <f>LEN(TRIM(D34))</f>
+        <f t="shared" ref="P34:P65" si="9">LEN(TRIM(D34))</f>
         <v>2</v>
       </c>
     </row>
@@ -5347,31 +5353,31 @@
         <v>223</v>
       </c>
       <c r="J35">
-        <f>MOD(E35+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>20000</v>
       </c>
       <c r="K35">
-        <f>MOD(G35+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>75000</v>
       </c>
       <c r="L35" t="str">
-        <f>_xlfn.CONCAT(TRIM($D35),TEXT(E35,"00000"),TEXT(H35,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EP0000089999</v>
       </c>
       <c r="M35" t="str">
-        <f>_xlfn.CONCAT(TRIM($D35),TEXT(F35,"00000"),TEXT(H35,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EP3999989999</v>
       </c>
       <c r="N35" t="str">
-        <f>_xlfn.CONCAT(TRIM($D35),TEXT(E35,"00000"),TEXT(G35,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EP0000060000</v>
       </c>
       <c r="O35" t="str">
-        <f>_xlfn.CONCAT(TRIM($D35),TEXT(F35,"00000"),TEXT(G35,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EP3999960000</v>
       </c>
       <c r="P35">
-        <f>LEN(TRIM(D35))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -5404,31 +5410,31 @@
         <v>223</v>
       </c>
       <c r="J36">
-        <f>MOD(E36+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>20000</v>
       </c>
       <c r="K36">
-        <f>MOD(G36+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>45000</v>
       </c>
       <c r="L36" t="str">
-        <f>_xlfn.CONCAT(TRIM($D36),TEXT(E36,"00000"),TEXT(H36,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EP0000059999</v>
       </c>
       <c r="M36" t="str">
-        <f>_xlfn.CONCAT(TRIM($D36),TEXT(F36,"00000"),TEXT(H36,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EP3999959999</v>
       </c>
       <c r="N36" t="str">
-        <f>_xlfn.CONCAT(TRIM($D36),TEXT(E36,"00000"),TEXT(G36,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EP0000030000</v>
       </c>
       <c r="O36" t="str">
-        <f>_xlfn.CONCAT(TRIM($D36),TEXT(F36,"00000"),TEXT(G36,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EP3999930000</v>
       </c>
       <c r="P36">
-        <f>LEN(TRIM(D36))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -5461,31 +5467,31 @@
         <v>223</v>
       </c>
       <c r="J37">
-        <f>MOD(E37+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>20000</v>
       </c>
       <c r="K37">
-        <f>MOD(G37+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>15000</v>
       </c>
       <c r="L37" t="str">
-        <f>_xlfn.CONCAT(TRIM($D37),TEXT(E37,"00000"),TEXT(H37,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EP0000029999</v>
       </c>
       <c r="M37" t="str">
-        <f>_xlfn.CONCAT(TRIM($D37),TEXT(F37,"00000"),TEXT(H37,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EP3999929999</v>
       </c>
       <c r="N37" t="str">
-        <f>_xlfn.CONCAT(TRIM($D37),TEXT(E37,"00000"),TEXT(G37,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EP0000000000</v>
       </c>
       <c r="O37" t="str">
-        <f>_xlfn.CONCAT(TRIM($D37),TEXT(F37,"00000"),TEXT(G37,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EP3999900000</v>
       </c>
       <c r="P37">
-        <f>LEN(TRIM(D37))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -5518,31 +5524,31 @@
         <v>223</v>
       </c>
       <c r="J38">
-        <f>MOD(E38+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>60000</v>
       </c>
       <c r="K38">
-        <f>MOD(G38+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>75000</v>
       </c>
       <c r="L38" t="str">
-        <f>_xlfn.CONCAT(TRIM($D38),TEXT(E38,"00000"),TEXT(H38,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EP4000089999</v>
       </c>
       <c r="M38" t="str">
-        <f>_xlfn.CONCAT(TRIM($D38),TEXT(F38,"00000"),TEXT(H38,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EP7999989999</v>
       </c>
       <c r="N38" t="str">
-        <f>_xlfn.CONCAT(TRIM($D38),TEXT(E38,"00000"),TEXT(G38,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EP4000060000</v>
       </c>
       <c r="O38" t="str">
-        <f>_xlfn.CONCAT(TRIM($D38),TEXT(F38,"00000"),TEXT(G38,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EP7999960000</v>
       </c>
       <c r="P38">
-        <f>LEN(TRIM(D38))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -5575,31 +5581,31 @@
         <v>223</v>
       </c>
       <c r="J39">
-        <f>MOD(E39+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>60000</v>
       </c>
       <c r="K39">
-        <f>MOD(G39+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>45000</v>
       </c>
       <c r="L39" t="str">
-        <f>_xlfn.CONCAT(TRIM($D39),TEXT(E39,"00000"),TEXT(H39,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EP4000059999</v>
       </c>
       <c r="M39" t="str">
-        <f>_xlfn.CONCAT(TRIM($D39),TEXT(F39,"00000"),TEXT(H39,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EP7999959999</v>
       </c>
       <c r="N39" t="str">
-        <f>_xlfn.CONCAT(TRIM($D39),TEXT(E39,"00000"),TEXT(G39,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EP4000030000</v>
       </c>
       <c r="O39" t="str">
-        <f>_xlfn.CONCAT(TRIM($D39),TEXT(F39,"00000"),TEXT(G39,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EP7999930000</v>
       </c>
       <c r="P39">
-        <f>LEN(TRIM(D39))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -5632,31 +5638,31 @@
         <v>223</v>
       </c>
       <c r="J40">
-        <f>MOD(E40+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>60000</v>
       </c>
       <c r="K40">
-        <f>MOD(G40+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>15000</v>
       </c>
       <c r="L40" t="str">
-        <f>_xlfn.CONCAT(TRIM($D40),TEXT(E40,"00000"),TEXT(H40,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EP4000029999</v>
       </c>
       <c r="M40" t="str">
-        <f>_xlfn.CONCAT(TRIM($D40),TEXT(F40,"00000"),TEXT(H40,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EP7999929999</v>
       </c>
       <c r="N40" t="str">
-        <f>_xlfn.CONCAT(TRIM($D40),TEXT(E40,"00000"),TEXT(G40,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EP4000000000</v>
       </c>
       <c r="O40" t="str">
-        <f>_xlfn.CONCAT(TRIM($D40),TEXT(F40,"00000"),TEXT(G40,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EP7999900000</v>
       </c>
       <c r="P40">
-        <f>LEN(TRIM(D40))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -5686,31 +5692,31 @@
         <v>225</v>
       </c>
       <c r="J41">
-        <f>MOD(E41+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>20000</v>
       </c>
       <c r="K41">
-        <f>MOD(G41+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>65000</v>
       </c>
       <c r="L41" t="str">
-        <f>_xlfn.CONCAT(TRIM($D41),TEXT(E41,"00000"),TEXT(H41,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EQ0000079999</v>
       </c>
       <c r="M41" t="str">
-        <f>_xlfn.CONCAT(TRIM($D41),TEXT(F41,"00000"),TEXT(H41,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EQ3999979999</v>
       </c>
       <c r="N41" t="str">
-        <f>_xlfn.CONCAT(TRIM($D41),TEXT(E41,"00000"),TEXT(G41,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EQ0000050000</v>
       </c>
       <c r="O41" t="str">
-        <f>_xlfn.CONCAT(TRIM($D41),TEXT(F41,"00000"),TEXT(G41,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EQ3999950000</v>
       </c>
       <c r="P41">
-        <f>LEN(TRIM(D41))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -5743,31 +5749,31 @@
         <v>225</v>
       </c>
       <c r="J42">
-        <f>MOD(E42+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>20000</v>
       </c>
       <c r="K42">
-        <f>MOD(G42+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>35000</v>
       </c>
       <c r="L42" t="str">
-        <f>_xlfn.CONCAT(TRIM($D42),TEXT(E42,"00000"),TEXT(H42,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EQ0000049999</v>
       </c>
       <c r="M42" t="str">
-        <f>_xlfn.CONCAT(TRIM($D42),TEXT(F42,"00000"),TEXT(H42,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EQ3999949999</v>
       </c>
       <c r="N42" t="str">
-        <f>_xlfn.CONCAT(TRIM($D42),TEXT(E42,"00000"),TEXT(G42,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EQ0000020000</v>
       </c>
       <c r="O42" t="str">
-        <f>_xlfn.CONCAT(TRIM($D42),TEXT(F42,"00000"),TEXT(G42,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EQ3999920000</v>
       </c>
       <c r="P42">
-        <f>LEN(TRIM(D42))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -5800,31 +5806,31 @@
         <v>225</v>
       </c>
       <c r="J43">
-        <f>MOD(E43+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>60000</v>
       </c>
       <c r="K43">
-        <f>MOD(G43+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>65000</v>
       </c>
       <c r="L43" t="str">
-        <f>_xlfn.CONCAT(TRIM($D43),TEXT(E43,"00000"),TEXT(H43,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EQ4000079999</v>
       </c>
       <c r="M43" t="str">
-        <f>_xlfn.CONCAT(TRIM($D43),TEXT(F43,"00000"),TEXT(H43,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EQ7999979999</v>
       </c>
       <c r="N43" t="str">
-        <f>_xlfn.CONCAT(TRIM($D43),TEXT(E43,"00000"),TEXT(G43,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EQ4000050000</v>
       </c>
       <c r="O43" t="str">
-        <f>_xlfn.CONCAT(TRIM($D43),TEXT(F43,"00000"),TEXT(G43,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EQ7999950000</v>
       </c>
       <c r="P43">
-        <f>LEN(TRIM(D43))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -5857,31 +5863,31 @@
         <v>225</v>
       </c>
       <c r="J44">
-        <f>MOD(E44+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>60000</v>
       </c>
       <c r="K44">
-        <f>MOD(G44+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>35000</v>
       </c>
       <c r="L44" t="str">
-        <f>_xlfn.CONCAT(TRIM($D44),TEXT(E44,"00000"),TEXT(H44,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>EQ4000049999</v>
       </c>
       <c r="M44" t="str">
-        <f>_xlfn.CONCAT(TRIM($D44),TEXT(F44,"00000"),TEXT(H44,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>EQ7999949999</v>
       </c>
       <c r="N44" t="str">
-        <f>_xlfn.CONCAT(TRIM($D44),TEXT(E44,"00000"),TEXT(G44,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>EQ4000020000</v>
       </c>
       <c r="O44" t="str">
-        <f>_xlfn.CONCAT(TRIM($D44),TEXT(F44,"00000"),TEXT(G44,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>EQ7999920000</v>
       </c>
       <c r="P44">
-        <f>LEN(TRIM(D44))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -5911,34 +5917,34 @@
         <v>99999</v>
       </c>
       <c r="I45" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="J45">
-        <f>MOD(E45+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>60000</v>
       </c>
       <c r="K45">
-        <f>MOD(G45+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>85000</v>
       </c>
       <c r="L45" t="str">
-        <f>_xlfn.CONCAT(TRIM($D45),TEXT(E45,"00000"),TEXT(H45,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>ER4000099999</v>
       </c>
       <c r="M45" t="str">
-        <f>_xlfn.CONCAT(TRIM($D45),TEXT(F45,"00000"),TEXT(H45,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>ER7999999999</v>
       </c>
       <c r="N45" t="str">
-        <f>_xlfn.CONCAT(TRIM($D45),TEXT(E45,"00000"),TEXT(G45,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>ER4000070000</v>
       </c>
       <c r="O45" t="str">
-        <f>_xlfn.CONCAT(TRIM($D45),TEXT(F45,"00000"),TEXT(G45,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>ER7999970000</v>
       </c>
       <c r="P45">
-        <f>LEN(TRIM(D45))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -5965,34 +5971,34 @@
         <v>59999</v>
       </c>
       <c r="I46" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J46">
-        <f>MOD(E46+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>20000</v>
       </c>
       <c r="K46">
-        <f>MOD(G46+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>45000</v>
       </c>
       <c r="L46" t="str">
-        <f>_xlfn.CONCAT(TRIM($D46),TEXT(E46,"00000"),TEXT(H46,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>ES0000059999</v>
       </c>
       <c r="M46" t="str">
-        <f>_xlfn.CONCAT(TRIM($D46),TEXT(F46,"00000"),TEXT(H46,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>ES3999959999</v>
       </c>
       <c r="N46" t="str">
-        <f>_xlfn.CONCAT(TRIM($D46),TEXT(E46,"00000"),TEXT(G46,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>ES0000030000</v>
       </c>
       <c r="O46" t="str">
-        <f>_xlfn.CONCAT(TRIM($D46),TEXT(F46,"00000"),TEXT(G46,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>ES3999930000</v>
       </c>
       <c r="P46">
-        <f>LEN(TRIM(D46))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -6022,34 +6028,34 @@
         <v>29999</v>
       </c>
       <c r="I47" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J47">
-        <f>MOD(E47+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>60000</v>
       </c>
       <c r="K47">
-        <f>MOD(G47+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>15000</v>
       </c>
       <c r="L47" t="str">
-        <f>_xlfn.CONCAT(TRIM($D47),TEXT(E47,"00000"),TEXT(H47,"00000"))</f>
+        <f t="shared" si="2"/>
         <v>ES4000029999</v>
       </c>
       <c r="M47" t="str">
-        <f>_xlfn.CONCAT(TRIM($D47),TEXT(F47,"00000"),TEXT(H47,"00000"))</f>
+        <f t="shared" si="3"/>
         <v>ES7999929999</v>
       </c>
       <c r="N47" t="str">
-        <f>_xlfn.CONCAT(TRIM($D47),TEXT(E47,"00000"),TEXT(G47,"00000"))</f>
+        <f t="shared" si="4"/>
         <v>ES4000000000</v>
       </c>
       <c r="O47" t="str">
-        <f>_xlfn.CONCAT(TRIM($D47),TEXT(F47,"00000"),TEXT(G47,"00000"))</f>
+        <f t="shared" si="5"/>
         <v>ES7999900000</v>
       </c>
       <c r="P47">
-        <f>LEN(TRIM(D47))</f>
+        <f t="shared" si="9"/>
         <v>2</v>
       </c>
     </row>
@@ -6079,14 +6085,14 @@
         <v>99999</v>
       </c>
       <c r="I48" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J48">
-        <f>MOD(E48+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K48">
-        <f>MOD(G48+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>85000</v>
       </c>
       <c r="L48" t="str">
@@ -6094,19 +6100,19 @@
         <v>CN8000099999</v>
       </c>
       <c r="M48" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D48),2),TEXT(F48,"00000"),TEXT(H48,"00000"))</f>
+        <f t="shared" ref="M48:M54" si="10">_xlfn.CONCAT(RIGHT(TRIM($D48),2),TEXT(F48,"00000"),TEXT(H48,"00000"))</f>
         <v>DN1999999999</v>
       </c>
       <c r="N48" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D48),2),TEXT(E48,"00000"),TEXT(G48,"00000"))</f>
+        <f t="shared" ref="N48:N54" si="11">_xlfn.CONCAT(LEFT(TRIM($D48),2),TEXT(E48,"00000"),TEXT(G48,"00000"))</f>
         <v>CN8000070000</v>
       </c>
       <c r="O48" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D48),2),TEXT(F48,"00000"),TEXT(G48,"00000"))</f>
+        <f t="shared" ref="O48:O73" si="12">_xlfn.CONCAT(RIGHT(TRIM($D48),2),TEXT(F48,"00000"),TEXT(G48,"00000"))</f>
         <v>DN1999970000</v>
       </c>
       <c r="P48">
-        <f>LEN(TRIM(D48))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q48" t="str">
@@ -6140,38 +6146,38 @@
         <v>69999</v>
       </c>
       <c r="I49" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J49">
-        <f>MOD(E49+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K49">
-        <f>MOD(G49+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>55000</v>
       </c>
       <c r="L49" t="str">
-        <f t="shared" ref="L49:L73" si="0">_xlfn.CONCAT(LEFT(TRIM($D49),2),TEXT(E49,"00000"),TEXT(H49,"00000"))</f>
+        <f t="shared" ref="L49:L73" si="13">_xlfn.CONCAT(LEFT(TRIM($D49),2),TEXT(E49,"00000"),TEXT(H49,"00000"))</f>
         <v>CN8000069999</v>
       </c>
       <c r="M49" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D49),2),TEXT(F49,"00000"),TEXT(H49,"00000"))</f>
+        <f t="shared" si="10"/>
         <v>DN1999969999</v>
       </c>
       <c r="N49" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D49),2),TEXT(E49,"00000"),TEXT(G49,"00000"))</f>
+        <f t="shared" si="11"/>
         <v>CN8000040000</v>
       </c>
       <c r="O49" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D49),2),TEXT(F49,"00000"),TEXT(G49,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>DN1999940000</v>
       </c>
       <c r="P49">
-        <f>LEN(TRIM(D49))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q49" t="str">
-        <f t="shared" ref="Q49:Q73" si="1">IF(F49&lt;E49,"Y","")</f>
+        <f t="shared" ref="Q49:Q73" si="14">IF(F49&lt;E49,"Y","")</f>
         <v>Y</v>
       </c>
     </row>
@@ -6204,35 +6210,35 @@
         <v>222</v>
       </c>
       <c r="J50">
-        <f>MOD(E50+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K50">
-        <f>MOD(G50+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>75000</v>
       </c>
       <c r="L50" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>CP8000089999</v>
       </c>
       <c r="M50" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D50),2),TEXT(F50,"00000"),TEXT(H50,"00000"))</f>
+        <f t="shared" si="10"/>
         <v>DP1999989999</v>
       </c>
       <c r="N50" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D50),2),TEXT(E50,"00000"),TEXT(G50,"00000"))</f>
+        <f t="shared" si="11"/>
         <v>CP8000060000</v>
       </c>
       <c r="O50" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D50),2),TEXT(F50,"00000"),TEXT(G50,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>DP1999960000</v>
       </c>
       <c r="P50">
-        <f>LEN(TRIM(D50))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q50" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -6265,35 +6271,35 @@
         <v>222</v>
       </c>
       <c r="J51">
-        <f>MOD(E51+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K51">
-        <f>MOD(G51+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>45000</v>
       </c>
       <c r="L51" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>CP8000059999</v>
       </c>
       <c r="M51" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D51),2),TEXT(F51,"00000"),TEXT(H51,"00000"))</f>
+        <f t="shared" si="10"/>
         <v>DP1999959999</v>
       </c>
       <c r="N51" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D51),2),TEXT(E51,"00000"),TEXT(G51,"00000"))</f>
+        <f t="shared" si="11"/>
         <v>CP8000030000</v>
       </c>
       <c r="O51" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D51),2),TEXT(F51,"00000"),TEXT(G51,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>DP1999930000</v>
       </c>
       <c r="P51">
-        <f>LEN(TRIM(D51))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q51" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -6326,35 +6332,35 @@
         <v>222</v>
       </c>
       <c r="J52">
-        <f>MOD(E52+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K52">
-        <f>MOD(G52+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>15000</v>
       </c>
       <c r="L52" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>CP8000029999</v>
       </c>
       <c r="M52" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D52),2),TEXT(F52,"00000"),TEXT(H52,"00000"))</f>
+        <f t="shared" si="10"/>
         <v>DP1999929999</v>
       </c>
       <c r="N52" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D52),2),TEXT(E52,"00000"),TEXT(G52,"00000"))</f>
+        <f t="shared" si="11"/>
         <v>CP8000000000</v>
       </c>
       <c r="O52" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D52),2),TEXT(F52,"00000"),TEXT(G52,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>DP1999900000</v>
       </c>
       <c r="P52">
-        <f>LEN(TRIM(D52))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q52" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -6387,35 +6393,35 @@
         <v>226</v>
       </c>
       <c r="J53">
-        <f>MOD(E53+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K53">
-        <f>MOD(G53+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>65000</v>
       </c>
       <c r="L53" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>CQ8000079999</v>
       </c>
       <c r="M53" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D53),2),TEXT(F53,"00000"),TEXT(H53,"00000"))</f>
+        <f t="shared" si="10"/>
         <v>DQ1999979999</v>
       </c>
       <c r="N53" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D53),2),TEXT(E53,"00000"),TEXT(G53,"00000"))</f>
+        <f t="shared" si="11"/>
         <v>CQ8000050000</v>
       </c>
       <c r="O53" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D53),2),TEXT(F53,"00000"),TEXT(G53,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>DQ1999950000</v>
       </c>
       <c r="P53">
-        <f>LEN(TRIM(D53))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q53" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -6448,35 +6454,35 @@
         <v>226</v>
       </c>
       <c r="J54">
-        <f>MOD(E54+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K54">
-        <f>MOD(G54+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>35000</v>
       </c>
       <c r="L54" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>CQ8000049999</v>
       </c>
       <c r="M54" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D54),2),TEXT(F54,"00000"),TEXT(H54,"00000"))</f>
+        <f t="shared" si="10"/>
         <v>DQ1999949999</v>
       </c>
       <c r="N54" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D54),2),TEXT(E54,"00000"),TEXT(G54,"00000"))</f>
+        <f t="shared" si="11"/>
         <v>CQ8000020000</v>
       </c>
       <c r="O54" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D54),2),TEXT(F54,"00000"),TEXT(G54,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>DQ1999920000</v>
       </c>
       <c r="P54">
-        <f>LEN(TRIM(D54))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q54" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -6491,7 +6497,7 @@
         <v>8211</v>
       </c>
       <c r="D55" t="s">
-        <v>228</v>
+        <v>251</v>
       </c>
       <c r="E55">
         <v>0</v>
@@ -6509,35 +6515,35 @@
         <v>220</v>
       </c>
       <c r="J55">
-        <f>MOD(E55+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>20000</v>
       </c>
       <c r="K55">
-        <f>MOD(G55+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>95000</v>
       </c>
       <c r="L55" t="str">
-        <f t="shared" si="0"/>
+        <f>_xlfn.CONCAT(RIGHT(TRIM($D55),2),TEXT(E55,"00000"),TEXT(H55,"00000"))</f>
         <v>EN0000009999</v>
       </c>
       <c r="M55" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D55),2),TEXT(F55,"00000"),TEXT(H55,"00000"))</f>
+        <f>_xlfn.CONCAT(RIGHT(TRIM($D55),2),TEXT(F55,"00000"),TEXT(H55,"00000"))</f>
         <v>EN3999909999</v>
       </c>
       <c r="N55" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D55),2),TEXT(E55,"00000"),TEXT(G55,"00000"))</f>
+        <f>_xlfn.CONCAT(LEFT(TRIM($D55),2),TEXT(E55,"00000"),TEXT(G55,"00000"))</f>
         <v>EM0000080000</v>
       </c>
       <c r="O55" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D55),2),TEXT(F55,"00000"),TEXT(G55,"00000"))</f>
+        <f>_xlfn.CONCAT(LEFT(TRIM($D55),2),TEXT(F55,"00000"),TEXT(G55,"00000"))</f>
         <v>EM3999980000</v>
       </c>
       <c r="P55">
-        <f>LEN(TRIM(D55))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q55" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
@@ -6567,38 +6573,38 @@
         <v>99999</v>
       </c>
       <c r="I56" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="J56">
-        <f>MOD(E56+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K56">
-        <f>MOD(G56+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>85000</v>
       </c>
       <c r="L56" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>EN8000099999</v>
       </c>
       <c r="M56" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D56),2),TEXT(F56,"00000"),TEXT(H56,"00000"))</f>
+        <f t="shared" ref="M56:M63" si="15">_xlfn.CONCAT(RIGHT(TRIM($D56),2),TEXT(F56,"00000"),TEXT(H56,"00000"))</f>
         <v>FN1999999999</v>
       </c>
       <c r="N56" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D56),2),TEXT(E56,"00000"),TEXT(G56,"00000"))</f>
+        <f t="shared" ref="N56:N63" si="16">_xlfn.CONCAT(LEFT(TRIM($D56),2),TEXT(E56,"00000"),TEXT(G56,"00000"))</f>
         <v>EN8000070000</v>
       </c>
       <c r="O56" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D56),2),TEXT(F56,"00000"),TEXT(G56,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>FN1999970000</v>
       </c>
       <c r="P56">
-        <f>LEN(TRIM(D56))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q56" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -6628,38 +6634,38 @@
         <v>89999</v>
       </c>
       <c r="I57" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="J57">
-        <f>MOD(E57+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K57">
-        <f>MOD(G57+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>75000</v>
       </c>
       <c r="L57" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>EP8000089999</v>
       </c>
       <c r="M57" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D57),2),TEXT(F57,"00000"),TEXT(H57,"00000"))</f>
+        <f t="shared" si="15"/>
         <v>FP1999989999</v>
       </c>
       <c r="N57" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D57),2),TEXT(E57,"00000"),TEXT(G57,"00000"))</f>
+        <f t="shared" si="16"/>
         <v>EP8000060000</v>
       </c>
       <c r="O57" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D57),2),TEXT(F57,"00000"),TEXT(G57,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>FP1999960000</v>
       </c>
       <c r="P57">
-        <f>LEN(TRIM(D57))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q57" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -6689,38 +6695,38 @@
         <v>59999</v>
       </c>
       <c r="I58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="J58">
-        <f>MOD(E58+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K58">
-        <f>MOD(G58+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>45000</v>
       </c>
       <c r="L58" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>EP8000059999</v>
       </c>
       <c r="M58" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D58),2),TEXT(F58,"00000"),TEXT(H58,"00000"))</f>
+        <f t="shared" si="15"/>
         <v>FP1999959999</v>
       </c>
       <c r="N58" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D58),2),TEXT(E58,"00000"),TEXT(G58,"00000"))</f>
+        <f t="shared" si="16"/>
         <v>EP8000030000</v>
       </c>
       <c r="O58" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D58),2),TEXT(F58,"00000"),TEXT(G58,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>FP1999930000</v>
       </c>
       <c r="P58">
-        <f>LEN(TRIM(D58))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q58" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -6750,38 +6756,38 @@
         <v>29999</v>
       </c>
       <c r="I59" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="J59">
-        <f>MOD(E59+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K59">
-        <f>MOD(G59+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>15000</v>
       </c>
       <c r="L59" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>EP8000029999</v>
       </c>
       <c r="M59" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D59),2),TEXT(F59,"00000"),TEXT(H59,"00000"))</f>
+        <f t="shared" si="15"/>
         <v>FP1999929999</v>
       </c>
       <c r="N59" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D59),2),TEXT(E59,"00000"),TEXT(G59,"00000"))</f>
+        <f t="shared" si="16"/>
         <v>EP8000000000</v>
       </c>
       <c r="O59" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D59),2),TEXT(F59,"00000"),TEXT(G59,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>FP1999900000</v>
       </c>
       <c r="P59">
-        <f>LEN(TRIM(D59))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q59" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -6811,38 +6817,38 @@
         <v>79999</v>
       </c>
       <c r="I60" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J60">
-        <f>MOD(E60+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K60">
-        <f>MOD(G60+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>65000</v>
       </c>
       <c r="L60" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>EQ8000079999</v>
       </c>
       <c r="M60" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D60),2),TEXT(F60,"00000"),TEXT(H60,"00000"))</f>
+        <f t="shared" si="15"/>
         <v>FQ1999979999</v>
       </c>
       <c r="N60" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D60),2),TEXT(E60,"00000"),TEXT(G60,"00000"))</f>
+        <f t="shared" si="16"/>
         <v>EQ8000050000</v>
       </c>
       <c r="O60" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D60),2),TEXT(F60,"00000"),TEXT(G60,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>FQ1999950000</v>
       </c>
       <c r="P60">
-        <f>LEN(TRIM(D60))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q60" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -6872,38 +6878,38 @@
         <v>49999</v>
       </c>
       <c r="I61" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J61">
-        <f>MOD(E61+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K61">
-        <f>MOD(G61+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>35000</v>
       </c>
       <c r="L61" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>EQ8000049999</v>
       </c>
       <c r="M61" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D61),2),TEXT(F61,"00000"),TEXT(H61,"00000"))</f>
+        <f t="shared" si="15"/>
         <v>FQ1999949999</v>
       </c>
       <c r="N61" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D61),2),TEXT(E61,"00000"),TEXT(G61,"00000"))</f>
+        <f t="shared" si="16"/>
         <v>EQ8000020000</v>
       </c>
       <c r="O61" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D61),2),TEXT(F61,"00000"),TEXT(G61,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>FQ1999920000</v>
       </c>
       <c r="P61">
-        <f>LEN(TRIM(D61))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q61" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -6933,38 +6939,38 @@
         <v>99999</v>
       </c>
       <c r="I62" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J62">
-        <f>MOD(E62+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K62">
-        <f>MOD(G62+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>85000</v>
       </c>
       <c r="L62" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>ER8000099999</v>
       </c>
       <c r="M62" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D62),2),TEXT(F62,"00000"),TEXT(H62,"00000"))</f>
+        <f t="shared" si="15"/>
         <v>FR1999999999</v>
       </c>
       <c r="N62" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D62),2),TEXT(E62,"00000"),TEXT(G62,"00000"))</f>
+        <f t="shared" si="16"/>
         <v>ER8000070000</v>
       </c>
       <c r="O62" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D62),2),TEXT(F62,"00000"),TEXT(G62,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>FR1999970000</v>
       </c>
       <c r="P62">
-        <f>LEN(TRIM(D62))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q62" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -6994,38 +7000,38 @@
         <v>39999</v>
       </c>
       <c r="I63" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J63">
-        <f>MOD(E63+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="K63">
-        <f>MOD(G63+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>25000</v>
       </c>
       <c r="L63" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="13"/>
         <v>ER8000039999</v>
       </c>
       <c r="M63" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D63),2),TEXT(F63,"00000"),TEXT(H63,"00000"))</f>
+        <f t="shared" si="15"/>
         <v>FR1999939999</v>
       </c>
       <c r="N63" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D63),2),TEXT(E63,"00000"),TEXT(G63,"00000"))</f>
+        <f t="shared" si="16"/>
         <v>ER8000010000</v>
       </c>
       <c r="O63" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D63),2),TEXT(F63,"00000"),TEXT(G63,"00000"))</f>
+        <f t="shared" si="12"/>
         <v>FR1999910000</v>
       </c>
       <c r="P63">
-        <f>LEN(TRIM(D63))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q63" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v>Y</v>
       </c>
     </row>
@@ -7055,35 +7061,35 @@
         <v>218</v>
       </c>
       <c r="J64">
-        <f>MOD(E64+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>20000</v>
       </c>
       <c r="K64">
-        <f>MOD(G64+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>95000</v>
       </c>
       <c r="L64" t="str">
-        <f t="shared" si="0"/>
-        <v>CQ0000009999</v>
+        <f>_xlfn.CONCAT(RIGHT(TRIM($D64),2),TEXT(E64,"00000"),TEXT(H64,"00000"))</f>
+        <v>CR0000009999</v>
       </c>
       <c r="M64" t="str">
-        <f>_xlfn.CONCAT(LEFT(TRIM($D64),2),TEXT(F64,"00000"),TEXT(H64,"00000"))</f>
-        <v>CQ3999909999</v>
+        <f>_xlfn.CONCAT(RIGHT(TRIM($D64),2),TEXT(F64,"00000"),TEXT(H64,"00000"))</f>
+        <v>CR3999909999</v>
       </c>
       <c r="N64" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D64),2),TEXT(E64,"00000"),TEXT(G64,"00000"))</f>
-        <v>CR0000080000</v>
+        <f>_xlfn.CONCAT(LEFT(TRIM($D64),2),TEXT(E64,"00000"),TEXT(G64,"00000"))</f>
+        <v>CQ0000080000</v>
       </c>
       <c r="O64" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D64),2),TEXT(F64,"00000"),TEXT(G64,"00000"))</f>
-        <v>CR3999980000</v>
+        <f>_xlfn.CONCAT(LEFT(TRIM($D64),2),TEXT(F64,"00000"),TEXT(G64,"00000"))</f>
+        <v>CQ3999980000</v>
       </c>
       <c r="P64">
-        <f>LEN(TRIM(D64))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q64" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
@@ -7116,35 +7122,35 @@
         <v>218</v>
       </c>
       <c r="J65">
-        <f>MOD(E65+20000,100000)</f>
+        <f t="shared" si="7"/>
         <v>20000</v>
       </c>
       <c r="K65">
-        <f>MOD(G65+15000,100000)</f>
+        <f t="shared" si="8"/>
         <v>5000</v>
       </c>
       <c r="L65" t="str">
-        <f t="shared" si="0"/>
-        <v>CP0000019999</v>
+        <f t="shared" ref="L65:L73" si="17">_xlfn.CONCAT(RIGHT(TRIM($D65),2),TEXT(E65,"00000"),TEXT(H65,"00000"))</f>
+        <v>CQ0000019999</v>
       </c>
       <c r="M65" t="str">
-        <f t="shared" ref="M65:M73" si="2">_xlfn.CONCAT(LEFT(TRIM($D65),2),TEXT(F65,"00000"),TEXT(H65,"00000"))</f>
-        <v>CP3999919999</v>
+        <f t="shared" ref="M65:M73" si="18">_xlfn.CONCAT(RIGHT(TRIM($D65),2),TEXT(F65,"00000"),TEXT(H65,"00000"))</f>
+        <v>CQ3999919999</v>
       </c>
       <c r="N65" t="str">
-        <f t="shared" ref="N65:N73" si="3">_xlfn.CONCAT(RIGHT(TRIM($D65),2),TEXT(E65,"00000"),TEXT(G65,"00000"))</f>
-        <v>CQ0000090000</v>
+        <f t="shared" ref="N65:N73" si="19">_xlfn.CONCAT(LEFT(TRIM($D65),2),TEXT(E65,"00000"),TEXT(G65,"00000"))</f>
+        <v>CP0000090000</v>
       </c>
       <c r="O65" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D65),2),TEXT(F65,"00000"),TEXT(G65,"00000"))</f>
-        <v>CQ3999990000</v>
+        <f t="shared" ref="O65:O73" si="20">_xlfn.CONCAT(LEFT(TRIM($D65),2),TEXT(F65,"00000"),TEXT(G65,"00000"))</f>
+        <v>CP3999990000</v>
       </c>
       <c r="P65">
-        <f>LEN(TRIM(D65))</f>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="Q65" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
@@ -7177,35 +7183,35 @@
         <v>225</v>
       </c>
       <c r="J66">
-        <f>MOD(E66+20000,100000)</f>
+        <f t="shared" ref="J66:J76" si="21">MOD(E66+20000,100000)</f>
         <v>20000</v>
       </c>
       <c r="K66">
-        <f>MOD(G66+15000,100000)</f>
+        <f t="shared" ref="K66:K76" si="22">MOD(G66+15000,100000)</f>
         <v>5000</v>
       </c>
       <c r="L66" t="str">
-        <f t="shared" si="0"/>
-        <v>EP0000019999</v>
+        <f t="shared" si="17"/>
+        <v>EQ0000019999</v>
       </c>
       <c r="M66" t="str">
-        <f t="shared" si="2"/>
-        <v>EP3999919999</v>
+        <f t="shared" si="18"/>
+        <v>EQ3999919999</v>
       </c>
       <c r="N66" t="str">
-        <f t="shared" si="3"/>
-        <v>EQ0000090000</v>
+        <f t="shared" si="19"/>
+        <v>EP0000090000</v>
       </c>
       <c r="O66" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D66),2),TEXT(F66,"00000"),TEXT(G66,"00000"))</f>
-        <v>EQ3999990000</v>
+        <f t="shared" si="20"/>
+        <v>EP3999990000</v>
       </c>
       <c r="P66">
-        <f>LEN(TRIM(D66))</f>
+        <f t="shared" ref="P66:P76" si="23">LEN(TRIM(D66))</f>
         <v>5</v>
       </c>
       <c r="Q66" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
@@ -7238,35 +7244,35 @@
         <v>225</v>
       </c>
       <c r="J67">
-        <f>MOD(E67+20000,100000)</f>
+        <f t="shared" si="21"/>
         <v>40000</v>
       </c>
       <c r="K67">
-        <f>MOD(G67+15000,100000)</f>
+        <f t="shared" si="22"/>
         <v>5000</v>
       </c>
       <c r="L67" t="str">
-        <f t="shared" si="0"/>
-        <v>DP2000019999</v>
+        <f t="shared" si="17"/>
+        <v>DQ2000019999</v>
       </c>
       <c r="M67" t="str">
-        <f t="shared" si="2"/>
-        <v>DP5999919999</v>
+        <f t="shared" si="18"/>
+        <v>DQ5999919999</v>
       </c>
       <c r="N67" t="str">
-        <f t="shared" si="3"/>
-        <v>DQ2000090000</v>
+        <f t="shared" si="19"/>
+        <v>DP2000090000</v>
       </c>
       <c r="O67" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D67),2),TEXT(F67,"00000"),TEXT(G67,"00000"))</f>
-        <v>DQ5999990000</v>
+        <f t="shared" si="20"/>
+        <v>DP5999990000</v>
       </c>
       <c r="P67">
-        <f>LEN(TRIM(D67))</f>
+        <f t="shared" si="23"/>
         <v>5</v>
       </c>
       <c r="Q67" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
@@ -7281,7 +7287,7 @@
         <v>8011</v>
       </c>
       <c r="D68" t="s">
-        <v>72</v>
+        <v>249</v>
       </c>
       <c r="E68">
         <v>20000</v>
@@ -7299,35 +7305,35 @@
         <v>221</v>
       </c>
       <c r="J68">
-        <f>MOD(E68+20000,100000)</f>
+        <f t="shared" si="21"/>
         <v>40000</v>
       </c>
       <c r="K68">
-        <f>MOD(G68+15000,100000)</f>
+        <f t="shared" si="22"/>
         <v>95000</v>
       </c>
       <c r="L68" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="17"/>
         <v>DN2000009999</v>
       </c>
       <c r="M68" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="18"/>
         <v>DN5999909999</v>
       </c>
       <c r="N68" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="19"/>
         <v>DM2000080000</v>
       </c>
       <c r="O68" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D68),2),TEXT(F68,"00000"),TEXT(G68,"00000"))</f>
+        <f t="shared" si="20"/>
         <v>DM5999980000</v>
       </c>
       <c r="P68">
-        <f>LEN(TRIM(D68))</f>
+        <f t="shared" si="23"/>
         <v>5</v>
       </c>
       <c r="Q68" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
@@ -7357,35 +7363,35 @@
         <v>225</v>
       </c>
       <c r="J69">
-        <f>MOD(E69+20000,100000)</f>
+        <f t="shared" si="21"/>
         <v>60000</v>
       </c>
       <c r="K69">
-        <f>MOD(G69+15000,100000)</f>
+        <f t="shared" si="22"/>
         <v>95000</v>
       </c>
       <c r="L69" t="str">
-        <f t="shared" si="0"/>
-        <v>EQ4000009999</v>
+        <f t="shared" si="17"/>
+        <v>ER4000009999</v>
       </c>
       <c r="M69" t="str">
-        <f t="shared" si="2"/>
-        <v>EQ7999909999</v>
+        <f t="shared" si="18"/>
+        <v>ER7999909999</v>
       </c>
       <c r="N69" t="str">
-        <f t="shared" si="3"/>
-        <v>ER4000080000</v>
+        <f t="shared" si="19"/>
+        <v>EQ4000080000</v>
       </c>
       <c r="O69" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D69),2),TEXT(F69,"00000"),TEXT(G69,"00000"))</f>
-        <v>ER7999980000</v>
+        <f t="shared" si="20"/>
+        <v>EQ7999980000</v>
       </c>
       <c r="P69">
-        <f>LEN(TRIM(D69))</f>
+        <f t="shared" si="23"/>
         <v>5</v>
       </c>
       <c r="Q69" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
@@ -7418,35 +7424,35 @@
         <v>218</v>
       </c>
       <c r="J70">
-        <f>MOD(E70+20000,100000)</f>
+        <f t="shared" si="21"/>
         <v>60000</v>
       </c>
       <c r="K70">
-        <f>MOD(G70+15000,100000)</f>
+        <f t="shared" si="22"/>
         <v>5000</v>
       </c>
       <c r="L70" t="str">
-        <f t="shared" si="0"/>
-        <v>CP4000019999</v>
+        <f t="shared" si="17"/>
+        <v>CQ4000019999</v>
       </c>
       <c r="M70" t="str">
-        <f t="shared" si="2"/>
-        <v>CP7999919999</v>
+        <f t="shared" si="18"/>
+        <v>CQ7999919999</v>
       </c>
       <c r="N70" t="str">
-        <f t="shared" si="3"/>
-        <v>CQ4000090000</v>
+        <f t="shared" si="19"/>
+        <v>CP4000090000</v>
       </c>
       <c r="O70" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D70),2),TEXT(F70,"00000"),TEXT(G70,"00000"))</f>
-        <v>CQ7999990000</v>
+        <f t="shared" si="20"/>
+        <v>CP7999990000</v>
       </c>
       <c r="P70">
-        <f>LEN(TRIM(D70))</f>
+        <f t="shared" si="23"/>
         <v>5</v>
       </c>
       <c r="Q70" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
@@ -7479,35 +7485,35 @@
         <v>225</v>
       </c>
       <c r="J71">
-        <f>MOD(E71+20000,100000)</f>
+        <f t="shared" si="21"/>
         <v>60000</v>
       </c>
       <c r="K71">
-        <f>MOD(G71+15000,100000)</f>
+        <f t="shared" si="22"/>
         <v>5000</v>
       </c>
       <c r="L71" t="str">
-        <f t="shared" si="0"/>
-        <v>EP4000019999</v>
+        <f t="shared" si="17"/>
+        <v>EQ4000019999</v>
       </c>
       <c r="M71" t="str">
-        <f t="shared" si="2"/>
-        <v>EP7999919999</v>
+        <f t="shared" si="18"/>
+        <v>EQ7999919999</v>
       </c>
       <c r="N71" t="str">
-        <f t="shared" si="3"/>
-        <v>EQ4000090000</v>
+        <f t="shared" si="19"/>
+        <v>EP4000090000</v>
       </c>
       <c r="O71" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D71),2),TEXT(F71,"00000"),TEXT(G71,"00000"))</f>
-        <v>EQ7999990000</v>
+        <f t="shared" si="20"/>
+        <v>EP7999990000</v>
       </c>
       <c r="P71">
-        <f>LEN(TRIM(D71))</f>
+        <f t="shared" si="23"/>
         <v>5</v>
       </c>
       <c r="Q71" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
@@ -7540,35 +7546,35 @@
         <v>226</v>
       </c>
       <c r="J72">
-        <f>MOD(E72+20000,100000)</f>
+        <f t="shared" si="21"/>
         <v>80000</v>
       </c>
       <c r="K72">
-        <f>MOD(G72+15000,100000)</f>
+        <f t="shared" si="22"/>
         <v>5000</v>
       </c>
       <c r="L72" t="str">
-        <f t="shared" si="0"/>
-        <v>DP6000019999</v>
+        <f t="shared" si="17"/>
+        <v>DQ6000019999</v>
       </c>
       <c r="M72" t="str">
-        <f t="shared" si="2"/>
-        <v>DP9999919999</v>
+        <f t="shared" si="18"/>
+        <v>DQ9999919999</v>
       </c>
       <c r="N72" t="str">
-        <f t="shared" si="3"/>
-        <v>DQ6000090000</v>
+        <f t="shared" si="19"/>
+        <v>DP6000090000</v>
       </c>
       <c r="O72" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D72),2),TEXT(F72,"00000"),TEXT(G72,"00000"))</f>
-        <v>DQ9999990000</v>
+        <f t="shared" si="20"/>
+        <v>DP9999990000</v>
       </c>
       <c r="P72">
-        <f>LEN(TRIM(D72))</f>
+        <f t="shared" si="23"/>
         <v>5</v>
       </c>
       <c r="Q72" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
@@ -7583,7 +7589,7 @@
         <v>8211</v>
       </c>
       <c r="D73" t="s">
-        <v>72</v>
+        <v>250</v>
       </c>
       <c r="E73">
         <v>60000</v>
@@ -7601,35 +7607,35 @@
         <v>221</v>
       </c>
       <c r="J73">
-        <f>MOD(E73+20000,100000)</f>
+        <f t="shared" si="21"/>
         <v>80000</v>
       </c>
       <c r="K73">
-        <f>MOD(G73+15000,100000)</f>
+        <f t="shared" si="22"/>
         <v>95000</v>
       </c>
       <c r="L73" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="17"/>
         <v>DN6000009999</v>
       </c>
       <c r="M73" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="18"/>
         <v>DN9999909999</v>
       </c>
       <c r="N73" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="19"/>
         <v>DM6000080000</v>
       </c>
       <c r="O73" t="str">
-        <f>_xlfn.CONCAT(RIGHT(TRIM($D73),2),TEXT(F73,"00000"),TEXT(G73,"00000"))</f>
+        <f t="shared" si="20"/>
         <v>DM9999980000</v>
       </c>
       <c r="P73">
-        <f>LEN(TRIM(D73))</f>
+        <f t="shared" si="23"/>
         <v>5</v>
       </c>
       <c r="Q73" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
@@ -7662,27 +7668,27 @@
         <v>221</v>
       </c>
       <c r="J74">
-        <f>MOD(E74+20000,100000)</f>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="K74">
-        <f>MOD(G74+15000,100000)</f>
+        <f t="shared" si="22"/>
         <v>95000</v>
       </c>
       <c r="L74" t="s">
+        <v>240</v>
+      </c>
+      <c r="M74" t="s">
         <v>241</v>
       </c>
-      <c r="M74" t="s">
-        <v>244</v>
-      </c>
       <c r="N74" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="O74" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="P74">
-        <f>LEN(TRIM(D74))</f>
+        <f t="shared" si="23"/>
         <v>11</v>
       </c>
     </row>
@@ -7715,27 +7721,27 @@
         <v>226</v>
       </c>
       <c r="J75">
-        <f>MOD(E75+20000,100000)</f>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="K75">
-        <f>MOD(G75+15000,100000)</f>
+        <f t="shared" si="22"/>
         <v>5000</v>
       </c>
       <c r="L75" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="M75" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="N75" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="O75" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="P75">
-        <f>LEN(TRIM(D75))</f>
+        <f t="shared" si="23"/>
         <v>11</v>
       </c>
     </row>
@@ -7765,30 +7771,30 @@
         <v>19999</v>
       </c>
       <c r="I76" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J76">
-        <f>MOD(E76+20000,100000)</f>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="K76">
-        <f>MOD(G76+15000,100000)</f>
+        <f t="shared" si="22"/>
         <v>5000</v>
       </c>
       <c r="L76" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="M76" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="N76" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="O76" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="P76">
-        <f>LEN(TRIM(D76))</f>
+        <f t="shared" si="23"/>
         <v>11</v>
       </c>
     </row>
@@ -7894,10 +7900,10 @@
         <v>219</v>
       </c>
       <c r="J6" t="s">
+        <v>228</v>
+      </c>
+      <c r="K6" t="s">
         <v>229</v>
-      </c>
-      <c r="K6" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
docs(spec): add gpx-tracks specification
</commit_message>
<xml_diff>
--- a/assets/tasmap50k.xlsx
+++ b/assets/tasmap50k.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrian/Development/mapping/peak_bagger/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A116002-100D-B34D-92F6-34FAA08EB4F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D71E3C-2C7F-3C4D-BAE4-518ED8DDB05E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1305,9 +1305,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -6006,7 +6008,7 @@
       <c r="A47" t="s">
         <v>117</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="2" t="s">
         <v>118</v>
       </c>
       <c r="C47">
@@ -6063,7 +6065,7 @@
       <c r="A48" t="s">
         <v>42</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="3" t="s">
         <v>43</v>
       </c>
       <c r="C48">
@@ -6108,7 +6110,7 @@
         <v>CN8000070000</v>
       </c>
       <c r="O48" t="str">
-        <f t="shared" ref="O48:O73" si="12">_xlfn.CONCAT(RIGHT(TRIM($D48),2),TEXT(F48,"00000"),TEXT(G48,"00000"))</f>
+        <f t="shared" ref="O48:O63" si="12">_xlfn.CONCAT(RIGHT(TRIM($D48),2),TEXT(F48,"00000"),TEXT(G48,"00000"))</f>
         <v>DN1999970000</v>
       </c>
       <c r="P48">
@@ -6124,7 +6126,7 @@
       <c r="A49" t="s">
         <v>45</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="3" t="s">
         <v>46</v>
       </c>
       <c r="C49">
@@ -6157,7 +6159,7 @@
         <v>55000</v>
       </c>
       <c r="L49" t="str">
-        <f t="shared" ref="L49:L73" si="13">_xlfn.CONCAT(LEFT(TRIM($D49),2),TEXT(E49,"00000"),TEXT(H49,"00000"))</f>
+        <f t="shared" ref="L49:L63" si="13">_xlfn.CONCAT(LEFT(TRIM($D49),2),TEXT(E49,"00000"),TEXT(H49,"00000"))</f>
         <v>CN8000069999</v>
       </c>
       <c r="M49" t="str">
@@ -6185,7 +6187,7 @@
       <c r="A50" t="s">
         <v>35</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="3" t="s">
         <v>36</v>
       </c>
       <c r="C50">
@@ -6490,7 +6492,7 @@
       <c r="A55" t="s">
         <v>114</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="2" t="s">
         <v>115</v>
       </c>
       <c r="C55">
@@ -6551,7 +6553,7 @@
       <c r="A56" t="s">
         <v>161</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="3" t="s">
         <v>162</v>
       </c>
       <c r="C56">
@@ -6917,7 +6919,7 @@
       <c r="A62" t="s">
         <v>141</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B62" s="3" t="s">
         <v>142</v>
       </c>
       <c r="C62">
@@ -7039,7 +7041,7 @@
       <c r="A64" t="s">
         <v>210</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B64" s="2" t="s">
         <v>211</v>
       </c>
       <c r="D64" t="s">
@@ -7097,7 +7099,7 @@
       <c r="A65" t="s">
         <v>13</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C65">
@@ -7158,7 +7160,7 @@
       <c r="A66" t="s">
         <v>97</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="2" t="s">
         <v>98</v>
       </c>
       <c r="C66">
@@ -7280,7 +7282,7 @@
       <c r="A68" t="s">
         <v>70</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="2" t="s">
         <v>71</v>
       </c>
       <c r="C68">
@@ -7582,7 +7584,7 @@
       <c r="A73" t="s">
         <v>92</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="2" t="s">
         <v>93</v>
       </c>
       <c r="C73">

</xml_diff>

<commit_message>
fix(app): refresh tasmap and admin views
</commit_message>
<xml_diff>
--- a/assets/tasmap50k.xlsx
+++ b/assets/tasmap50k.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrian/Development/mapping/peak_bagger/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DA95DA2-888B-A040-9862-60CEA129CBCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9006D64F-6925-5C47-A75F-378038AEDDFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1751,12 +1751,6 @@
     <t>DN 19999 39999</t>
   </si>
   <si>
-    <t>DM 19999 32000</t>
-  </si>
-  <si>
-    <t>CM 90000 32000</t>
-  </si>
-  <si>
     <t>EN 60000 40000</t>
   </si>
   <si>
@@ -1767,6 +1761,12 @@
   </si>
   <si>
     <t>EN 51000 40000</t>
+  </si>
+  <si>
+    <t>DM 19999 80000</t>
+  </si>
+  <si>
+    <t>CM 90000 80000</t>
   </si>
 </sst>
 </file>
@@ -3969,16 +3969,16 @@
         <v>395</v>
       </c>
       <c r="O27" t="s">
-        <v>575</v>
+        <v>570</v>
       </c>
       <c r="P27" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="Q27" t="s">
+        <v>572</v>
+      </c>
+      <c r="R27" t="s">
         <v>573</v>
-      </c>
-      <c r="R27" t="s">
-        <v>572</v>
       </c>
       <c r="S27" t="s">
         <v>394</v>
@@ -5303,10 +5303,10 @@
         <v>569</v>
       </c>
       <c r="N55" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="O55" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="AF55" t="s">
         <v>247</v>

</xml_diff>

<commit_message>
feat(tasmap): add display mode cycling
</commit_message>
<xml_diff>
--- a/assets/tasmap50k.xlsx
+++ b/assets/tasmap50k.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrian/Development/mapping/peak_bagger/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9006D64F-6925-5C47-A75F-378038AEDDFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{351800FA-1677-0741-A7D7-47591BBD9DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="569">
   <si>
     <t>Series</t>
   </si>
@@ -782,42 +782,6 @@
     <t>northingMid</t>
   </si>
   <si>
-    <t>CN9039</t>
-  </si>
-  <si>
-    <t>DN1939</t>
-  </si>
-  <si>
-    <t>CM9098</t>
-  </si>
-  <si>
-    <t>DM1998</t>
-  </si>
-  <si>
-    <t>DM1185</t>
-  </si>
-  <si>
-    <t>DM1197</t>
-  </si>
-  <si>
-    <t>DM1997</t>
-  </si>
-  <si>
-    <t>DM1985</t>
-  </si>
-  <si>
-    <t>DM3239</t>
-  </si>
-  <si>
-    <t>DM8939</t>
-  </si>
-  <si>
-    <t>DM8432</t>
-  </si>
-  <si>
-    <t>DM8932</t>
-  </si>
-  <si>
     <t>BQ 98000 79999</t>
   </si>
   <si>
@@ -1625,15 +1589,9 @@
     <t>EP7999900000</t>
   </si>
   <si>
-    <t>CQ8000079999</t>
-  </si>
-  <si>
     <t>DQ1999979999</t>
   </si>
   <si>
-    <t>CQ8000050000</t>
-  </si>
-  <si>
     <t>DQ1999950000</t>
   </si>
   <si>
@@ -1745,9 +1703,6 @@
     <t>p8</t>
   </si>
   <si>
-    <t>CN 90000 39999</t>
-  </si>
-  <si>
     <t>DN 19999 39999</t>
   </si>
   <si>
@@ -1763,10 +1718,34 @@
     <t>EN 51000 40000</t>
   </si>
   <si>
-    <t>DM 19999 80000</t>
-  </si>
-  <si>
     <t>CM 90000 80000</t>
+  </si>
+  <si>
+    <t>CN 84000 39999</t>
+  </si>
+  <si>
+    <t>DM 19999 85000</t>
+  </si>
+  <si>
+    <t>DM 11000 85000</t>
+  </si>
+  <si>
+    <t>DM 11000 98000</t>
+  </si>
+  <si>
+    <t>CM 90000 98000</t>
+  </si>
+  <si>
+    <t>CN 90000 32000</t>
+  </si>
+  <si>
+    <t>CN 84000 32000</t>
+  </si>
+  <si>
+    <t>CQ7000079999</t>
+  </si>
+  <si>
+    <t>CQ7000050000</t>
   </si>
 </sst>
 </file>
@@ -2691,7 +2670,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AQ76"/>
+  <dimension ref="A1:S76"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
@@ -2741,28 +2720,28 @@
         <v>246</v>
       </c>
       <c r="L1" t="s">
-        <v>560</v>
+        <v>546</v>
       </c>
       <c r="M1" t="s">
-        <v>561</v>
+        <v>547</v>
       </c>
       <c r="N1" t="s">
-        <v>562</v>
+        <v>548</v>
       </c>
       <c r="O1" t="s">
-        <v>563</v>
+        <v>549</v>
       </c>
       <c r="P1" t="s">
-        <v>564</v>
+        <v>550</v>
       </c>
       <c r="Q1" t="s">
-        <v>565</v>
+        <v>551</v>
       </c>
       <c r="R1" t="s">
-        <v>566</v>
+        <v>552</v>
       </c>
       <c r="S1" t="s">
-        <v>567</v>
+        <v>553</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
@@ -2800,16 +2779,16 @@
         <v>95000</v>
       </c>
       <c r="L2" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
       <c r="M2" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
       <c r="N2" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="O2" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
@@ -2847,16 +2826,16 @@
         <v>25000</v>
       </c>
       <c r="L3" t="s">
-        <v>300</v>
+        <v>288</v>
       </c>
       <c r="M3" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="N3" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
       <c r="O3" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
@@ -2894,16 +2873,16 @@
         <v>75000</v>
       </c>
       <c r="L4" t="s">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="M4" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="N4" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="O4" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
@@ -2941,16 +2920,16 @@
         <v>85000</v>
       </c>
       <c r="L5" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="M5" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="N5" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="O5" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
@@ -2985,16 +2964,16 @@
         <v>95000</v>
       </c>
       <c r="L6" t="s">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="M6" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="N6" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="O6" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
@@ -3032,16 +3011,16 @@
         <v>95000</v>
       </c>
       <c r="L7" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="M7" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="N7" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="O7" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
@@ -3079,16 +3058,16 @@
         <v>35000</v>
       </c>
       <c r="L8" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="M8" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="N8" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="O8" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
@@ -3126,16 +3105,16 @@
         <v>5000</v>
       </c>
       <c r="L9" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="M9" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="N9" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="O9" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
@@ -3220,16 +3199,16 @@
         <v>15000</v>
       </c>
       <c r="L11" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="M11" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="N11" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="O11" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
@@ -3267,16 +3246,16 @@
         <v>65000</v>
       </c>
       <c r="L12" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="M12" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="N12" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
       <c r="O12" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
@@ -3311,16 +3290,16 @@
         <v>95000</v>
       </c>
       <c r="L13" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="M13" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="N13" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="O13" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
@@ -3358,16 +3337,16 @@
         <v>75000</v>
       </c>
       <c r="L14" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="M14" t="s">
-        <v>341</v>
+        <v>329</v>
       </c>
       <c r="N14" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="O14" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.2">
@@ -3402,16 +3381,16 @@
         <v>15000</v>
       </c>
       <c r="L15" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="M15" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
       <c r="N15" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
       <c r="O15" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
@@ -3446,16 +3425,16 @@
         <v>55000</v>
       </c>
       <c r="L16" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="M16" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="N16" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="O16" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
@@ -3493,16 +3472,16 @@
         <v>25000</v>
       </c>
       <c r="L17" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
       <c r="M17" t="s">
-        <v>353</v>
+        <v>341</v>
       </c>
       <c r="N17" t="s">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="O17" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
@@ -3537,16 +3516,16 @@
         <v>65000</v>
       </c>
       <c r="L18" t="s">
-        <v>356</v>
+        <v>344</v>
       </c>
       <c r="M18" t="s">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="N18" t="s">
-        <v>359</v>
+        <v>347</v>
       </c>
       <c r="O18" t="s">
-        <v>358</v>
+        <v>346</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.2">
@@ -3584,16 +3563,16 @@
         <v>35000</v>
       </c>
       <c r="L19" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="M19" t="s">
-        <v>361</v>
+        <v>349</v>
       </c>
       <c r="N19" t="s">
-        <v>363</v>
+        <v>351</v>
       </c>
       <c r="O19" t="s">
-        <v>362</v>
+        <v>350</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.2">
@@ -3631,16 +3610,16 @@
         <v>85000</v>
       </c>
       <c r="L20" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="M20" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="N20" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="O20" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.2">
@@ -3678,16 +3657,16 @@
         <v>45000</v>
       </c>
       <c r="L21" t="s">
-        <v>368</v>
+        <v>356</v>
       </c>
       <c r="M21" t="s">
-        <v>369</v>
+        <v>357</v>
       </c>
       <c r="N21" t="s">
-        <v>371</v>
+        <v>359</v>
       </c>
       <c r="O21" t="s">
-        <v>370</v>
+        <v>358</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.2">
@@ -3725,16 +3704,16 @@
         <v>55000</v>
       </c>
       <c r="L22" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="M22" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
       <c r="N22" t="s">
-        <v>375</v>
+        <v>363</v>
       </c>
       <c r="O22" t="s">
-        <v>374</v>
+        <v>362</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.2">
@@ -3772,16 +3751,16 @@
         <v>75000</v>
       </c>
       <c r="L23" t="s">
-        <v>376</v>
+        <v>364</v>
       </c>
       <c r="M23" t="s">
-        <v>377</v>
+        <v>365</v>
       </c>
       <c r="N23" t="s">
-        <v>379</v>
+        <v>367</v>
       </c>
       <c r="O23" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.2">
@@ -3819,16 +3798,16 @@
         <v>45000</v>
       </c>
       <c r="L24" t="s">
-        <v>380</v>
+        <v>368</v>
       </c>
       <c r="M24" t="s">
-        <v>381</v>
+        <v>369</v>
       </c>
       <c r="N24" t="s">
-        <v>383</v>
+        <v>371</v>
       </c>
       <c r="O24" t="s">
-        <v>382</v>
+        <v>370</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.2">
@@ -3866,16 +3845,16 @@
         <v>35000</v>
       </c>
       <c r="L25" t="s">
-        <v>384</v>
+        <v>372</v>
       </c>
       <c r="M25" t="s">
-        <v>385</v>
+        <v>373</v>
       </c>
       <c r="N25" t="s">
-        <v>387</v>
+        <v>375</v>
       </c>
       <c r="O25" t="s">
-        <v>386</v>
+        <v>374</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.2">
@@ -3913,16 +3892,16 @@
         <v>5000</v>
       </c>
       <c r="L26" t="s">
-        <v>388</v>
+        <v>376</v>
       </c>
       <c r="M26" t="s">
-        <v>389</v>
+        <v>377</v>
       </c>
       <c r="N26" t="s">
-        <v>391</v>
+        <v>379</v>
       </c>
       <c r="O26" t="s">
-        <v>390</v>
+        <v>378</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.2">
@@ -3960,28 +3939,28 @@
         <v>55000</v>
       </c>
       <c r="L27" t="s">
-        <v>392</v>
+        <v>380</v>
       </c>
       <c r="M27" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="N27" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="O27" t="s">
-        <v>570</v>
+        <v>555</v>
       </c>
       <c r="P27" t="s">
-        <v>571</v>
+        <v>556</v>
       </c>
       <c r="Q27" t="s">
-        <v>572</v>
+        <v>557</v>
       </c>
       <c r="R27" t="s">
-        <v>573</v>
+        <v>558</v>
       </c>
       <c r="S27" t="s">
-        <v>394</v>
+        <v>382</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.2">
@@ -4019,16 +3998,16 @@
         <v>15000</v>
       </c>
       <c r="L28" t="s">
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="M28" t="s">
-        <v>397</v>
+        <v>385</v>
       </c>
       <c r="N28" t="s">
-        <v>399</v>
+        <v>387</v>
       </c>
       <c r="O28" t="s">
-        <v>398</v>
+        <v>386</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.2">
@@ -4066,16 +4045,16 @@
         <v>15000</v>
       </c>
       <c r="L29" t="s">
-        <v>400</v>
+        <v>388</v>
       </c>
       <c r="M29" t="s">
-        <v>401</v>
+        <v>389</v>
       </c>
       <c r="N29" t="s">
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="O29" t="s">
-        <v>402</v>
+        <v>390</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
@@ -4113,16 +4092,16 @@
         <v>85000</v>
       </c>
       <c r="L30" t="s">
-        <v>404</v>
+        <v>392</v>
       </c>
       <c r="M30" t="s">
-        <v>405</v>
+        <v>393</v>
       </c>
       <c r="N30" t="s">
-        <v>407</v>
+        <v>395</v>
       </c>
       <c r="O30" t="s">
-        <v>406</v>
+        <v>394</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.2">
@@ -4160,16 +4139,16 @@
         <v>25000</v>
       </c>
       <c r="L31" t="s">
-        <v>408</v>
+        <v>396</v>
       </c>
       <c r="M31" t="s">
-        <v>409</v>
+        <v>397</v>
       </c>
       <c r="N31" t="s">
-        <v>411</v>
+        <v>399</v>
       </c>
       <c r="O31" t="s">
-        <v>410</v>
+        <v>398</v>
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.2">
@@ -4204,28 +4183,28 @@
         <v>69000</v>
       </c>
       <c r="L32" t="s">
-        <v>291</v>
+        <v>279</v>
       </c>
       <c r="M32" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
       <c r="N32" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="O32" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="P32" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="Q32" t="s">
-        <v>288</v>
+        <v>276</v>
       </c>
       <c r="R32" t="s">
-        <v>289</v>
+        <v>277</v>
       </c>
       <c r="S32" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
@@ -4263,16 +4242,16 @@
         <v>75000</v>
       </c>
       <c r="L33" t="s">
-        <v>412</v>
+        <v>400</v>
       </c>
       <c r="M33" t="s">
-        <v>413</v>
+        <v>401</v>
       </c>
       <c r="N33" t="s">
-        <v>415</v>
+        <v>403</v>
       </c>
       <c r="O33" t="s">
-        <v>414</v>
+        <v>402</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.2">
@@ -4310,16 +4289,16 @@
         <v>75000</v>
       </c>
       <c r="L34" t="s">
-        <v>416</v>
+        <v>404</v>
       </c>
       <c r="M34" t="s">
-        <v>417</v>
+        <v>405</v>
       </c>
       <c r="N34" t="s">
-        <v>419</v>
+        <v>407</v>
       </c>
       <c r="O34" t="s">
-        <v>418</v>
+        <v>406</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.2">
@@ -4354,16 +4333,16 @@
         <v>45000</v>
       </c>
       <c r="L35" t="s">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="M35" t="s">
-        <v>421</v>
+        <v>409</v>
       </c>
       <c r="N35" t="s">
-        <v>423</v>
+        <v>411</v>
       </c>
       <c r="O35" t="s">
-        <v>422</v>
+        <v>410</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.2">
@@ -4401,16 +4380,16 @@
         <v>15000</v>
       </c>
       <c r="L36" t="s">
-        <v>424</v>
+        <v>412</v>
       </c>
       <c r="M36" t="s">
-        <v>425</v>
+        <v>413</v>
       </c>
       <c r="N36" t="s">
-        <v>427</v>
+        <v>415</v>
       </c>
       <c r="O36" t="s">
-        <v>426</v>
+        <v>414</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.2">
@@ -4448,16 +4427,16 @@
         <v>45000</v>
       </c>
       <c r="L37" t="s">
-        <v>428</v>
+        <v>416</v>
       </c>
       <c r="M37" t="s">
-        <v>429</v>
+        <v>417</v>
       </c>
       <c r="N37" t="s">
-        <v>431</v>
+        <v>419</v>
       </c>
       <c r="O37" t="s">
-        <v>430</v>
+        <v>418</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.2">
@@ -4495,16 +4474,16 @@
         <v>55000</v>
       </c>
       <c r="L38" t="s">
-        <v>432</v>
+        <v>420</v>
       </c>
       <c r="M38" t="s">
-        <v>433</v>
+        <v>421</v>
       </c>
       <c r="N38" t="s">
-        <v>435</v>
+        <v>423</v>
       </c>
       <c r="O38" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.2">
@@ -4542,16 +4521,16 @@
         <v>75000</v>
       </c>
       <c r="L39" t="s">
-        <v>436</v>
+        <v>424</v>
       </c>
       <c r="M39" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
       <c r="N39" t="s">
-        <v>439</v>
+        <v>427</v>
       </c>
       <c r="O39" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.2">
@@ -4589,16 +4568,16 @@
         <v>35000</v>
       </c>
       <c r="L40" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
       <c r="M40" t="s">
-        <v>441</v>
+        <v>429</v>
       </c>
       <c r="N40" t="s">
-        <v>443</v>
+        <v>431</v>
       </c>
       <c r="O40" t="s">
-        <v>442</v>
+        <v>430</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.2">
@@ -4636,16 +4615,16 @@
         <v>15000</v>
       </c>
       <c r="L41" t="s">
-        <v>444</v>
+        <v>432</v>
       </c>
       <c r="M41" t="s">
-        <v>445</v>
+        <v>433</v>
       </c>
       <c r="N41" t="s">
-        <v>447</v>
+        <v>435</v>
       </c>
       <c r="O41" t="s">
-        <v>446</v>
+        <v>434</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.2">
@@ -4683,16 +4662,16 @@
         <v>85000</v>
       </c>
       <c r="L42" t="s">
-        <v>448</v>
+        <v>436</v>
       </c>
       <c r="M42" t="s">
-        <v>449</v>
+        <v>437</v>
       </c>
       <c r="N42" t="s">
-        <v>451</v>
+        <v>439</v>
       </c>
       <c r="O42" t="s">
-        <v>450</v>
+        <v>438</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.2">
@@ -4730,16 +4709,16 @@
         <v>85000</v>
       </c>
       <c r="L43" t="s">
-        <v>452</v>
+        <v>440</v>
       </c>
       <c r="M43" t="s">
-        <v>453</v>
+        <v>441</v>
       </c>
       <c r="N43" t="s">
-        <v>455</v>
+        <v>443</v>
       </c>
       <c r="O43" t="s">
-        <v>454</v>
+        <v>442</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.2">
@@ -4777,16 +4756,16 @@
         <v>5000</v>
       </c>
       <c r="L44" t="s">
-        <v>456</v>
+        <v>444</v>
       </c>
       <c r="M44" t="s">
-        <v>457</v>
+        <v>445</v>
       </c>
       <c r="N44" t="s">
-        <v>459</v>
+        <v>447</v>
       </c>
       <c r="O44" t="s">
-        <v>458</v>
+        <v>446</v>
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.2">
@@ -4800,7 +4779,7 @@
         <v>7916</v>
       </c>
       <c r="D45" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="E45">
         <v>98000</v>
@@ -4824,16 +4803,16 @@
         <v>65000</v>
       </c>
       <c r="L45" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="M45" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="N45" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="O45" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.2">
@@ -4871,16 +4850,16 @@
         <v>45000</v>
       </c>
       <c r="L46" t="s">
-        <v>460</v>
+        <v>448</v>
       </c>
       <c r="M46" t="s">
-        <v>461</v>
+        <v>449</v>
       </c>
       <c r="N46" t="s">
-        <v>463</v>
+        <v>451</v>
       </c>
       <c r="O46" t="s">
-        <v>462</v>
+        <v>450</v>
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.2">
@@ -4918,16 +4897,16 @@
         <v>65000</v>
       </c>
       <c r="L47" t="s">
-        <v>464</v>
+        <v>452</v>
       </c>
       <c r="M47" t="s">
-        <v>465</v>
+        <v>453</v>
       </c>
       <c r="N47" t="s">
-        <v>467</v>
+        <v>455</v>
       </c>
       <c r="O47" t="s">
-        <v>466</v>
+        <v>454</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.2">
@@ -4965,19 +4944,19 @@
         <v>75000</v>
       </c>
       <c r="L48" t="s">
-        <v>468</v>
+        <v>456</v>
       </c>
       <c r="M48" t="s">
-        <v>469</v>
+        <v>457</v>
       </c>
       <c r="N48" t="s">
-        <v>471</v>
+        <v>459</v>
       </c>
       <c r="O48" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="49" spans="1:43" x14ac:dyDescent="0.2">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>145</v>
       </c>
@@ -5024,7 +5003,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="50" spans="1:43" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>193</v>
       </c>
@@ -5056,19 +5035,19 @@
         <v>65000</v>
       </c>
       <c r="L50" t="s">
-        <v>472</v>
+        <v>460</v>
       </c>
       <c r="M50" t="s">
-        <v>473</v>
+        <v>461</v>
       </c>
       <c r="N50" t="s">
-        <v>475</v>
+        <v>463</v>
       </c>
       <c r="O50" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="51" spans="1:43" x14ac:dyDescent="0.2">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>9</v>
       </c>
@@ -5103,25 +5082,25 @@
         <v>42000</v>
       </c>
       <c r="L51" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="M51" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="N51" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="O51" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="P51" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="Q51" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="52" spans="1:43" x14ac:dyDescent="0.2">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>46</v>
       </c>
@@ -5156,19 +5135,19 @@
         <v>35000</v>
       </c>
       <c r="L52" t="s">
-        <v>476</v>
+        <v>464</v>
       </c>
       <c r="M52" t="s">
-        <v>477</v>
+        <v>465</v>
       </c>
       <c r="N52" t="s">
-        <v>479</v>
+        <v>467</v>
       </c>
       <c r="O52" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="53" spans="1:43" x14ac:dyDescent="0.2">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>77</v>
       </c>
@@ -5203,19 +5182,19 @@
         <v>45000</v>
       </c>
       <c r="L53" t="s">
-        <v>480</v>
+        <v>468</v>
       </c>
       <c r="M53" t="s">
-        <v>481</v>
+        <v>469</v>
       </c>
       <c r="N53" t="s">
-        <v>483</v>
+        <v>471</v>
       </c>
       <c r="O53" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="54" spans="1:43" x14ac:dyDescent="0.2">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>92</v>
       </c>
@@ -5250,23 +5229,26 @@
         <v>5000</v>
       </c>
       <c r="L54" t="s">
-        <v>484</v>
+        <v>472</v>
       </c>
       <c r="M54" t="s">
-        <v>485</v>
+        <v>473</v>
       </c>
       <c r="N54" t="s">
-        <v>487</v>
+        <v>475</v>
       </c>
       <c r="O54" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="55" spans="1:43" x14ac:dyDescent="0.2">
+        <v>474</v>
+      </c>
+      <c r="P54" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>43</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="B55" s="4" t="s">
         <v>44</v>
       </c>
       <c r="C55">
@@ -5297,55 +5279,31 @@
         <v>54000</v>
       </c>
       <c r="L55" t="s">
-        <v>568</v>
+        <v>560</v>
       </c>
       <c r="M55" t="s">
-        <v>569</v>
+        <v>554</v>
       </c>
       <c r="N55" t="s">
-        <v>574</v>
+        <v>561</v>
       </c>
       <c r="O55" t="s">
-        <v>575</v>
-      </c>
-      <c r="AF55" t="s">
-        <v>247</v>
-      </c>
-      <c r="AG55" t="s">
-        <v>248</v>
-      </c>
-      <c r="AH55" t="s">
-        <v>249</v>
-      </c>
-      <c r="AI55" t="s">
-        <v>250</v>
-      </c>
-      <c r="AJ55" t="s">
-        <v>252</v>
-      </c>
-      <c r="AK55" t="s">
-        <v>253</v>
-      </c>
-      <c r="AL55" t="s">
-        <v>251</v>
-      </c>
-      <c r="AM55" t="s">
-        <v>254</v>
-      </c>
-      <c r="AN55" t="s">
-        <v>255</v>
-      </c>
-      <c r="AO55" t="s">
-        <v>256</v>
-      </c>
-      <c r="AP55" t="s">
-        <v>257</v>
-      </c>
-      <c r="AQ55" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="56" spans="1:43" x14ac:dyDescent="0.2">
+        <v>562</v>
+      </c>
+      <c r="P55" t="s">
+        <v>563</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>564</v>
+      </c>
+      <c r="R55" t="s">
+        <v>565</v>
+      </c>
+      <c r="S55" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>114</v>
       </c>
@@ -5380,19 +5338,19 @@
         <v>85000</v>
       </c>
       <c r="L56" t="s">
-        <v>488</v>
+        <v>476</v>
       </c>
       <c r="M56" t="s">
-        <v>489</v>
+        <v>477</v>
       </c>
       <c r="N56" t="s">
-        <v>491</v>
+        <v>479</v>
       </c>
       <c r="O56" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="57" spans="1:43" x14ac:dyDescent="0.2">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="57" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>38</v>
       </c>
@@ -5427,19 +5385,19 @@
         <v>85000</v>
       </c>
       <c r="L57" t="s">
-        <v>492</v>
+        <v>480</v>
       </c>
       <c r="M57" t="s">
-        <v>493</v>
+        <v>481</v>
       </c>
       <c r="N57" t="s">
-        <v>495</v>
+        <v>483</v>
       </c>
       <c r="O57" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="58" spans="1:43" x14ac:dyDescent="0.2">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="58" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>129</v>
       </c>
@@ -5474,19 +5432,19 @@
         <v>85000</v>
       </c>
       <c r="L58" t="s">
-        <v>496</v>
+        <v>484</v>
       </c>
       <c r="M58" t="s">
-        <v>497</v>
+        <v>485</v>
       </c>
       <c r="N58" t="s">
-        <v>499</v>
+        <v>487</v>
       </c>
       <c r="O58" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="59" spans="1:43" x14ac:dyDescent="0.2">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="59" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>12</v>
       </c>
@@ -5521,19 +5479,19 @@
         <v>35000</v>
       </c>
       <c r="L59" t="s">
-        <v>500</v>
+        <v>488</v>
       </c>
       <c r="M59" t="s">
-        <v>501</v>
+        <v>489</v>
       </c>
       <c r="N59" t="s">
-        <v>503</v>
+        <v>491</v>
       </c>
       <c r="O59" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="60" spans="1:43" x14ac:dyDescent="0.2">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="60" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>7</v>
       </c>
@@ -5568,19 +5526,19 @@
         <v>35000</v>
       </c>
       <c r="L60" t="s">
-        <v>504</v>
+        <v>492</v>
       </c>
       <c r="M60" t="s">
-        <v>505</v>
+        <v>493</v>
       </c>
       <c r="N60" t="s">
-        <v>507</v>
+        <v>495</v>
       </c>
       <c r="O60" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="61" spans="1:43" x14ac:dyDescent="0.2">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="61" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>89</v>
       </c>
@@ -5615,19 +5573,19 @@
         <v>35000</v>
       </c>
       <c r="L61" t="s">
-        <v>508</v>
+        <v>496</v>
       </c>
       <c r="M61" t="s">
-        <v>509</v>
+        <v>497</v>
       </c>
       <c r="N61" t="s">
-        <v>511</v>
+        <v>499</v>
       </c>
       <c r="O61" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="62" spans="1:43" x14ac:dyDescent="0.2">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="62" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>83</v>
       </c>
@@ -5662,19 +5620,19 @@
         <v>55000</v>
       </c>
       <c r="L62" t="s">
-        <v>512</v>
+        <v>500</v>
       </c>
       <c r="M62" t="s">
-        <v>513</v>
+        <v>501</v>
       </c>
       <c r="N62" t="s">
-        <v>515</v>
+        <v>503</v>
       </c>
       <c r="O62" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="63" spans="1:43" x14ac:dyDescent="0.2">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="63" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>109</v>
       </c>
@@ -5709,19 +5667,19 @@
         <v>95000</v>
       </c>
       <c r="L63" t="s">
-        <v>516</v>
+        <v>504</v>
       </c>
       <c r="M63" t="s">
-        <v>517</v>
+        <v>505</v>
       </c>
       <c r="N63" t="s">
-        <v>519</v>
+        <v>507</v>
       </c>
       <c r="O63" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="64" spans="1:43" x14ac:dyDescent="0.2">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="64" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>68</v>
       </c>
@@ -5756,22 +5714,22 @@
         <v>72000</v>
       </c>
       <c r="L64" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="M64" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
       <c r="N64" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="O64" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="P64" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="Q64" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
     </row>
     <row r="65" spans="1:19" x14ac:dyDescent="0.2">
@@ -5809,16 +5767,16 @@
         <v>45000</v>
       </c>
       <c r="L65" t="s">
-        <v>520</v>
+        <v>508</v>
       </c>
       <c r="M65" t="s">
-        <v>521</v>
+        <v>509</v>
       </c>
       <c r="N65" t="s">
-        <v>523</v>
+        <v>511</v>
       </c>
       <c r="O65" t="s">
-        <v>522</v>
+        <v>510</v>
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.2">
@@ -5856,16 +5814,16 @@
         <v>15000</v>
       </c>
       <c r="L66" t="s">
-        <v>524</v>
+        <v>512</v>
       </c>
       <c r="M66" t="s">
-        <v>525</v>
+        <v>513</v>
       </c>
       <c r="N66" t="s">
-        <v>527</v>
+        <v>515</v>
       </c>
       <c r="O66" t="s">
-        <v>526</v>
+        <v>514</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.2">
@@ -5903,16 +5861,16 @@
         <v>65000</v>
       </c>
       <c r="L67" t="s">
-        <v>528</v>
+        <v>567</v>
       </c>
       <c r="M67" t="s">
-        <v>529</v>
+        <v>516</v>
       </c>
       <c r="N67" t="s">
-        <v>531</v>
+        <v>517</v>
       </c>
       <c r="O67" t="s">
-        <v>530</v>
+        <v>568</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.2">
@@ -5950,28 +5908,28 @@
         <v>28500</v>
       </c>
       <c r="L68" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
       <c r="M68" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="N68" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
       <c r="O68" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="P68" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="Q68" t="s">
-        <v>294</v>
+        <v>282</v>
       </c>
       <c r="R68" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="S68" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
     </row>
     <row r="69" spans="1:19" x14ac:dyDescent="0.2">
@@ -6006,16 +5964,16 @@
         <v>71000</v>
       </c>
       <c r="L69" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="M69" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="N69" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="O69" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.2">
@@ -6050,16 +6008,16 @@
         <v>25000</v>
       </c>
       <c r="L70" t="s">
-        <v>532</v>
+        <v>518</v>
       </c>
       <c r="M70" t="s">
-        <v>533</v>
+        <v>519</v>
       </c>
       <c r="N70" t="s">
-        <v>535</v>
+        <v>521</v>
       </c>
       <c r="O70" t="s">
-        <v>534</v>
+        <v>520</v>
       </c>
     </row>
     <row r="71" spans="1:19" x14ac:dyDescent="0.2">
@@ -6097,16 +6055,16 @@
         <v>15000</v>
       </c>
       <c r="L71" t="s">
-        <v>536</v>
+        <v>522</v>
       </c>
       <c r="M71" t="s">
-        <v>537</v>
+        <v>523</v>
       </c>
       <c r="N71" t="s">
-        <v>539</v>
+        <v>525</v>
       </c>
       <c r="O71" t="s">
-        <v>538</v>
+        <v>524</v>
       </c>
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.2">
@@ -6144,16 +6102,16 @@
         <v>45000</v>
       </c>
       <c r="L72" t="s">
-        <v>540</v>
+        <v>526</v>
       </c>
       <c r="M72" t="s">
-        <v>541</v>
+        <v>527</v>
       </c>
       <c r="N72" t="s">
-        <v>543</v>
+        <v>529</v>
       </c>
       <c r="O72" t="s">
-        <v>542</v>
+        <v>528</v>
       </c>
     </row>
     <row r="73" spans="1:19" x14ac:dyDescent="0.2">
@@ -6191,16 +6149,16 @@
         <v>15000</v>
       </c>
       <c r="L73" t="s">
-        <v>544</v>
+        <v>530</v>
       </c>
       <c r="M73" t="s">
-        <v>545</v>
+        <v>531</v>
       </c>
       <c r="N73" t="s">
-        <v>547</v>
+        <v>533</v>
       </c>
       <c r="O73" t="s">
-        <v>546</v>
+        <v>532</v>
       </c>
     </row>
     <row r="74" spans="1:19" x14ac:dyDescent="0.2">
@@ -6238,16 +6196,16 @@
         <v>55000</v>
       </c>
       <c r="L74" t="s">
-        <v>548</v>
+        <v>534</v>
       </c>
       <c r="M74" t="s">
-        <v>549</v>
+        <v>535</v>
       </c>
       <c r="N74" t="s">
-        <v>551</v>
+        <v>537</v>
       </c>
       <c r="O74" t="s">
-        <v>550</v>
+        <v>536</v>
       </c>
     </row>
     <row r="75" spans="1:19" x14ac:dyDescent="0.2">
@@ -6285,16 +6243,16 @@
         <v>25000</v>
       </c>
       <c r="L75" t="s">
-        <v>552</v>
+        <v>538</v>
       </c>
       <c r="M75" t="s">
-        <v>553</v>
+        <v>539</v>
       </c>
       <c r="N75" t="s">
-        <v>555</v>
+        <v>541</v>
       </c>
       <c r="O75" t="s">
-        <v>554</v>
+        <v>540</v>
       </c>
     </row>
     <row r="76" spans="1:19" x14ac:dyDescent="0.2">
@@ -6332,16 +6290,16 @@
         <v>5000</v>
       </c>
       <c r="L76" t="s">
-        <v>556</v>
+        <v>542</v>
       </c>
       <c r="M76" t="s">
-        <v>557</v>
+        <v>543</v>
       </c>
       <c r="N76" t="s">
-        <v>559</v>
+        <v>545</v>
       </c>
       <c r="O76" t="s">
-        <v>558</v>
+        <v>544</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add peak list import and refresh services
</commit_message>
<xml_diff>
--- a/assets/tasmap50k.xlsx
+++ b/assets/tasmap50k.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrian/Development/mapping/peak_bagger/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{351800FA-1677-0741-A7D7-47591BBD9DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60397FD6-C302-644B-8A1C-8EEB3A5AD83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="569">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="568">
   <si>
     <t>Series</t>
   </si>
@@ -1716,9 +1716,6 @@
   </si>
   <si>
     <t>EN 51000 40000</t>
-  </si>
-  <si>
-    <t>CM 90000 80000</t>
   </si>
   <si>
     <t>CN 84000 39999</t>
@@ -5240,9 +5237,6 @@
       <c r="O54" t="s">
         <v>474</v>
       </c>
-      <c r="P54" t="s">
-        <v>559</v>
-      </c>
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
@@ -5279,28 +5273,28 @@
         <v>54000</v>
       </c>
       <c r="L55" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="M55" t="s">
         <v>554</v>
       </c>
       <c r="N55" t="s">
+        <v>560</v>
+      </c>
+      <c r="O55" t="s">
         <v>561</v>
       </c>
-      <c r="O55" t="s">
+      <c r="P55" t="s">
         <v>562</v>
       </c>
-      <c r="P55" t="s">
+      <c r="Q55" t="s">
         <v>563</v>
       </c>
-      <c r="Q55" t="s">
+      <c r="R55" t="s">
         <v>564</v>
       </c>
-      <c r="R55" t="s">
+      <c r="S55" t="s">
         <v>565</v>
-      </c>
-      <c r="S55" t="s">
-        <v>566</v>
       </c>
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.2">
@@ -5861,7 +5855,7 @@
         <v>65000</v>
       </c>
       <c r="L67" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="M67" t="s">
         <v>516</v>
@@ -5870,7 +5864,7 @@
         <v>517</v>
       </c>
       <c r="O67" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.2">

</xml_diff>